<commit_message>
small edit in police chauki
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/police chauki.xlsx
+++ b/बजेट माग estimate/police chauki.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB354258-E17A-4E2D-9919-450104364759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18D42E1-AA93-40BB-AC38-5E32F4AE5403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Estimate (4)" sheetId="10" r:id="rId1"/>
+    <sheet name="Estimate (4)" sheetId="10" state="hidden" r:id="rId1"/>
+    <sheet name="Police sector contribution" sheetId="11" r:id="rId2"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
+    <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
     <definedName name="description_103">[1]Abstract!$B$16</definedName>
     <definedName name="description_124" localSheetId="0">#REF!</definedName>
+    <definedName name="description_124" localSheetId="1">#REF!</definedName>
     <definedName name="description_124">#REF!</definedName>
     <definedName name="description_247">[1]Abstract!$B$22</definedName>
     <definedName name="description_248">[1]Abstract!$B$23</definedName>
@@ -31,6 +33,7 @@
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Estimate (4)'!$A$5:$K$66</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Police sector contribution'!$A$5:$K$66</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="46">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -183,6 +186,9 @@
   </si>
   <si>
     <t>Random Rubble Masonry, Providing and laying of Stone Masonry Work in Cement Mortar 1:6 in Foundation complete as per Drawing and Technical Specifications.</t>
+  </si>
+  <si>
+    <t>Police sector contribution</t>
   </si>
 </sst>
 </file>
@@ -368,7 +374,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -386,29 +392,28 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -419,7 +424,7 @@
     <xf numFmtId="2" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -428,26 +433,22 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -462,29 +463,17 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -549,7 +538,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -643,7 +632,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -702,9 +691,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -742,9 +731,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -777,26 +766,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -829,26 +801,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1037,113 +992,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="54"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="47"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="55" t="s">
+      <c r="A5" s="48" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="55"/>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="55"/>
-      <c r="G5" s="55"/>
-      <c r="H5" s="55"/>
-      <c r="I5" s="55"/>
-      <c r="J5" s="55"/>
-      <c r="K5" s="55"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="48"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+      <c r="K5" s="48"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
+      <c r="B6" s="51"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
       <c r="G6" s="1"/>
-      <c r="H6" s="59" t="s">
+      <c r="H6" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="59"/>
-      <c r="J6" s="59"/>
-      <c r="K6" s="59"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="60" t="s">
+      <c r="A7" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="60"/>
-      <c r="C7" s="60"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
+      <c r="B7" s="53"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="53"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="61" t="s">
+      <c r="H7" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61"/>
-      <c r="K7" s="61"/>
+      <c r="I7" s="54"/>
+      <c r="J7" s="54"/>
+      <c r="K7" s="54"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -1180,1158 +1135,1158 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" s="8" customFormat="1" ht="150" x14ac:dyDescent="0.25">
-      <c r="A9" s="33">
+    <row r="9" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+      <c r="A9" s="30">
         <v>1</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="32"/>
-      <c r="J9" s="32"/>
-      <c r="K9" s="32"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="33"/>
-      <c r="B10" s="34" t="s">
+      <c r="A10" s="30"/>
+      <c r="B10" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="32">
         <v>1</v>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="33">
         <f>65-D11*C11</f>
         <v>57.65</v>
       </c>
-      <c r="E10" s="36">
+      <c r="E10" s="33">
         <v>0.3</v>
       </c>
-      <c r="F10" s="36">
+      <c r="F10" s="33">
         <v>0.75</v>
       </c>
-      <c r="G10" s="36">
+      <c r="G10" s="33">
         <f>PRODUCT(C10:F10)</f>
         <v>12.971249999999998</v>
       </c>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="20"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="33"/>
-      <c r="B11" s="34"/>
-      <c r="C11" s="35">
+      <c r="A11" s="30"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="32">
         <v>21</v>
       </c>
-      <c r="D11" s="36">
+      <c r="D11" s="33">
         <v>0.35</v>
       </c>
-      <c r="E11" s="36">
+      <c r="E11" s="33">
         <v>0.35</v>
       </c>
-      <c r="F11" s="36">
+      <c r="F11" s="33">
         <v>1.75</v>
       </c>
-      <c r="G11" s="36">
+      <c r="G11" s="33">
         <f>PRODUCT(C11:F11)</f>
         <v>4.5018750000000001</v>
       </c>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="33"/>
-      <c r="B12" s="34" t="s">
+      <c r="A12" s="30"/>
+      <c r="B12" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="35">
+      <c r="C12" s="32">
         <v>1</v>
       </c>
-      <c r="D12" s="36">
+      <c r="D12" s="33">
         <v>58</v>
       </c>
-      <c r="E12" s="36">
+      <c r="E12" s="33">
         <f>1.5/2</f>
         <v>0.75</v>
       </c>
-      <c r="F12" s="36">
+      <c r="F12" s="33">
         <v>1.2</v>
       </c>
-      <c r="G12" s="36">
+      <c r="G12" s="33">
         <f>PRODUCT(C12:F12)</f>
         <v>52.199999999999996</v>
       </c>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="21"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
     </row>
     <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9"/>
-      <c r="B13" s="10" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="14">
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="13">
         <f>SUM(G10:G12)</f>
         <v>69.673124999999999</v>
       </c>
-      <c r="H13" s="15" t="s">
+      <c r="H13" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I13" s="14">
+      <c r="I13" s="13">
         <v>62.95</v>
       </c>
-      <c r="J13" s="16">
+      <c r="J13" s="15">
         <f>G13*I13</f>
         <v>4385.9232187500002</v>
       </c>
-      <c r="K13" s="13"/>
+      <c r="K13" s="12"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="33"/>
-      <c r="B14" s="37" t="s">
+      <c r="A14" s="30"/>
+      <c r="B14" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="16">
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="15">
         <f>0.13*G13*18612/360</f>
         <v>468.27307312499994</v>
       </c>
-      <c r="K14" s="21"/>
+      <c r="K14" s="20"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="33"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="21"/>
-    </row>
-    <row r="16" spans="1:11" s="8" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A16" s="33">
+      <c r="A15" s="30"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+    </row>
+    <row r="16" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A16" s="30">
         <v>2</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32"/>
-      <c r="J16" s="32"/>
-      <c r="K16" s="32"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="33"/>
-      <c r="B17" s="34" t="str">
+      <c r="A17" s="30"/>
+      <c r="B17" s="31" t="str">
         <f>B12</f>
         <v>-for  stone masonary</v>
       </c>
-      <c r="C17" s="35">
+      <c r="C17" s="32">
         <v>1</v>
       </c>
-      <c r="D17" s="36">
+      <c r="D17" s="33">
         <f>D12</f>
         <v>58</v>
       </c>
-      <c r="E17" s="36">
+      <c r="E17" s="33">
         <f>1.5/2</f>
         <v>0.75</v>
       </c>
-      <c r="F17" s="36">
+      <c r="F17" s="33">
         <v>0.15</v>
       </c>
-      <c r="G17" s="36">
+      <c r="G17" s="33">
         <f>PRODUCT(C17:F17)</f>
         <v>6.5249999999999995</v>
       </c>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
     </row>
     <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="9"/>
-      <c r="B18" s="10" t="s">
+      <c r="A18" s="8"/>
+      <c r="B18" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="14">
+      <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="13">
         <f>SUM(G17:G17)</f>
         <v>6.5249999999999995</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="H18" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I18" s="14">
+      <c r="I18" s="13">
         <v>4585.53</v>
       </c>
-      <c r="J18" s="16">
+      <c r="J18" s="15">
         <f>G18*I18</f>
         <v>29920.583249999996</v>
       </c>
-      <c r="K18" s="13"/>
+      <c r="K18" s="12"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="33"/>
-      <c r="B19" s="37" t="s">
+      <c r="A19" s="30"/>
+      <c r="B19" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="21"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="16">
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="15">
         <f>0.13*G18*15452.64/5</f>
         <v>2621.5403759999999</v>
       </c>
-      <c r="K19" s="21"/>
+      <c r="K19" s="20"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="33"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
+      <c r="A20" s="30"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="20"/>
     </row>
     <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="33">
+      <c r="A21" s="30">
         <v>3</v>
       </c>
-      <c r="B21" s="38" t="s">
+      <c r="B21" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="20"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="33"/>
-      <c r="B22" s="34" t="str">
+      <c r="A22" s="30"/>
+      <c r="B22" s="31" t="str">
         <f>B10</f>
         <v>-for brick wall</v>
       </c>
-      <c r="C22" s="35">
+      <c r="C22" s="32">
         <v>1</v>
       </c>
-      <c r="D22" s="36">
+      <c r="D22" s="33">
         <f>D10</f>
         <v>57.65</v>
       </c>
-      <c r="E22" s="36">
+      <c r="E22" s="33">
         <v>0.23</v>
       </c>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36">
+      <c r="F22" s="33"/>
+      <c r="G22" s="33">
         <f>PRODUCT(C22:F22)</f>
         <v>13.259500000000001</v>
       </c>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="33"/>
-      <c r="B23" s="34"/>
-      <c r="C23" s="35">
+      <c r="A23" s="30"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="32">
         <f>C11</f>
         <v>21</v>
       </c>
-      <c r="D23" s="36">
+      <c r="D23" s="33">
         <f>D11</f>
         <v>0.35</v>
       </c>
-      <c r="E23" s="36">
+      <c r="E23" s="33">
         <f>E11</f>
         <v>0.35</v>
       </c>
-      <c r="F23" s="36"/>
-      <c r="G23" s="36">
+      <c r="F23" s="33"/>
+      <c r="G23" s="33">
         <f>PRODUCT(C23:F23)</f>
         <v>2.5724999999999998</v>
       </c>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
     </row>
     <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9"/>
-      <c r="B24" s="10" t="s">
+      <c r="A24" s="8"/>
+      <c r="B24" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="14">
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="13">
         <f>SUM(G22:G23)</f>
         <v>15.832000000000001</v>
       </c>
-      <c r="H24" s="15" t="s">
+      <c r="H24" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I24" s="14">
+      <c r="I24" s="13">
         <v>1017.47</v>
       </c>
-      <c r="J24" s="16">
+      <c r="J24" s="15">
         <f>G24*I24</f>
         <v>16108.585040000002</v>
       </c>
-      <c r="K24" s="13"/>
+      <c r="K24" s="12"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="33"/>
-      <c r="B25" s="37" t="s">
+      <c r="A25" s="30"/>
+      <c r="B25" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="16">
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="15">
         <f>0.13*G24*8617.2/10</f>
         <v>1773.5576352</v>
       </c>
-      <c r="K25" s="21"/>
+      <c r="K25" s="20"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="33"/>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
-      <c r="I26" s="21"/>
-      <c r="J26" s="21"/>
-      <c r="K26" s="21"/>
-    </row>
-    <row r="27" spans="1:11" s="8" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A27" s="33">
+      <c r="A26" s="30"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="20"/>
+    </row>
+    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A27" s="30">
         <v>4</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="32"/>
-      <c r="J27" s="32"/>
-      <c r="K27" s="32"/>
-    </row>
-    <row r="28" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="33"/>
-      <c r="B28" s="34" t="str">
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
+      <c r="I27" s="20"/>
+      <c r="J27" s="20"/>
+      <c r="K27" s="20"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="30"/>
+      <c r="B28" s="31" t="str">
         <f>B10</f>
         <v>-for brick wall</v>
       </c>
-      <c r="C28" s="32">
+      <c r="C28" s="20">
         <v>1</v>
       </c>
-      <c r="D28" s="39">
+      <c r="D28" s="36">
         <f>D10</f>
         <v>57.65</v>
       </c>
-      <c r="E28" s="32">
+      <c r="E28" s="20">
         <v>0.23</v>
       </c>
-      <c r="F28" s="36">
+      <c r="F28" s="33">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G28" s="36">
+      <c r="G28" s="33">
         <f t="shared" ref="G28:G33" si="0">PRODUCT(C28:F28)</f>
         <v>0.99446250000000003</v>
       </c>
-      <c r="H28" s="32"/>
-      <c r="I28" s="32"/>
-      <c r="J28" s="32"/>
-      <c r="K28" s="32"/>
-    </row>
-    <row r="29" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="33"/>
-      <c r="B29" s="34"/>
-      <c r="C29" s="32">
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="30"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="20">
         <v>2</v>
       </c>
-      <c r="D29" s="39">
+      <c r="D29" s="36">
         <f>D10</f>
         <v>57.65</v>
       </c>
-      <c r="E29" s="32">
+      <c r="E29" s="20">
         <v>0.23</v>
       </c>
-      <c r="F29" s="36">
+      <c r="F29" s="33">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G29" s="36">
+      <c r="G29" s="33">
         <f t="shared" si="0"/>
         <v>1.9889250000000001</v>
       </c>
-      <c r="H29" s="32"/>
-      <c r="I29" s="32"/>
-      <c r="J29" s="32"/>
-      <c r="K29" s="32"/>
-    </row>
-    <row r="30" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="33"/>
-      <c r="B30" s="34"/>
-      <c r="C30" s="32">
+      <c r="H29" s="20"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="20"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="30"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="20">
         <f>C11</f>
         <v>21</v>
       </c>
-      <c r="D30" s="39">
+      <c r="D30" s="36">
         <f>D11</f>
         <v>0.35</v>
       </c>
-      <c r="E30" s="39">
+      <c r="E30" s="36">
         <f>E11</f>
         <v>0.35</v>
       </c>
-      <c r="F30" s="39">
+      <c r="F30" s="36">
         <v>0.05</v>
       </c>
-      <c r="G30" s="36">
+      <c r="G30" s="33">
         <f t="shared" si="0"/>
         <v>0.12862499999999999</v>
       </c>
-      <c r="H30" s="32"/>
-      <c r="I30" s="32"/>
-      <c r="J30" s="32"/>
-      <c r="K30" s="32"/>
-    </row>
-    <row r="31" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="33"/>
-      <c r="B31" s="34"/>
-      <c r="C31" s="32">
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="20"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="30"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="20">
         <f>21*2</f>
         <v>42</v>
       </c>
-      <c r="D31" s="39">
+      <c r="D31" s="36">
         <v>0.35</v>
       </c>
-      <c r="E31" s="39">
+      <c r="E31" s="36">
         <v>0.35</v>
       </c>
-      <c r="F31" s="39">
+      <c r="F31" s="36">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G31" s="36">
+      <c r="G31" s="33">
         <f t="shared" si="0"/>
         <v>0.38587499999999997</v>
       </c>
-      <c r="H31" s="32"/>
-      <c r="I31" s="32"/>
-      <c r="J31" s="32"/>
-      <c r="K31" s="32"/>
+      <c r="H31" s="20"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="33"/>
-      <c r="B32" s="34" t="str">
+      <c r="A32" s="30"/>
+      <c r="B32" s="31" t="str">
         <f>B12</f>
         <v>-for  stone masonary</v>
       </c>
-      <c r="C32" s="35">
+      <c r="C32" s="32">
         <v>1</v>
       </c>
-      <c r="D32" s="36">
+      <c r="D32" s="33">
         <f>D12</f>
         <v>58</v>
       </c>
-      <c r="E32" s="36">
+      <c r="E32" s="33">
         <f>F53/2</f>
         <v>0.75</v>
       </c>
-      <c r="F32" s="36">
+      <c r="F32" s="33">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G32" s="36">
+      <c r="G32" s="33">
         <f t="shared" si="0"/>
         <v>3.2624999999999997</v>
       </c>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21"/>
+      <c r="H32" s="20"/>
+      <c r="I32" s="20"/>
+      <c r="J32" s="20"/>
+      <c r="K32" s="20"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="33"/>
-      <c r="B33" s="34"/>
-      <c r="C33" s="35">
+      <c r="A33" s="30"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="32">
         <v>1</v>
       </c>
-      <c r="D33" s="36">
+      <c r="D33" s="33">
         <f>D32</f>
         <v>58</v>
       </c>
-      <c r="E33" s="36">
+      <c r="E33" s="33">
         <v>0.45</v>
       </c>
-      <c r="F33" s="36">
+      <c r="F33" s="33">
         <v>0.05</v>
       </c>
-      <c r="G33" s="36">
+      <c r="G33" s="33">
         <f t="shared" si="0"/>
         <v>1.3050000000000002</v>
       </c>
-      <c r="H33" s="21"/>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
-      <c r="K33" s="21"/>
+      <c r="H33" s="20"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="20"/>
+      <c r="K33" s="20"/>
     </row>
     <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="9"/>
-      <c r="B34" s="10" t="s">
+      <c r="A34" s="8"/>
+      <c r="B34" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="11"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="14">
+      <c r="C34" s="10"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="13">
         <f>SUM(G28:G33)</f>
         <v>8.0653874999999999</v>
       </c>
-      <c r="H34" s="15" t="s">
+      <c r="H34" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I34" s="14">
+      <c r="I34" s="13">
         <v>10964.46</v>
       </c>
-      <c r="J34" s="16">
+      <c r="J34" s="15">
         <f>G34*I34</f>
         <v>88432.618628249998</v>
       </c>
-      <c r="K34" s="13"/>
+      <c r="K34" s="12"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="33"/>
-      <c r="B35" s="37" t="s">
+      <c r="A35" s="30"/>
+      <c r="B35" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-      <c r="G35" s="21"/>
-      <c r="H35" s="21"/>
-      <c r="I35" s="21"/>
-      <c r="J35" s="16">
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="20"/>
+      <c r="I35" s="20"/>
+      <c r="J35" s="15">
         <f>0.13*G34*(119450.3+6325.7)/15</f>
         <v>8791.7455444000007</v>
       </c>
-      <c r="K35" s="21"/>
+      <c r="K35" s="20"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="33"/>
-      <c r="B36" s="21"/>
-      <c r="C36" s="21"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="21"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="21"/>
-      <c r="J36" s="21"/>
-      <c r="K36" s="21"/>
+      <c r="A36" s="30"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="20"/>
+      <c r="I36" s="20"/>
+      <c r="J36" s="20"/>
+      <c r="K36" s="20"/>
     </row>
     <row r="37" spans="1:11" ht="32.25" x14ac:dyDescent="0.25">
-      <c r="A37" s="33">
+      <c r="A37" s="30">
         <v>5</v>
       </c>
-      <c r="B37" s="38" t="s">
+      <c r="B37" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="21"/>
-      <c r="G37" s="21"/>
-      <c r="H37" s="21"/>
-      <c r="I37" s="21"/>
-      <c r="J37" s="21"/>
-      <c r="K37" s="21"/>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="20"/>
+      <c r="I37" s="20"/>
+      <c r="J37" s="20"/>
+      <c r="K37" s="20"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" s="33"/>
-      <c r="B38" s="34" t="str">
+      <c r="A38" s="30"/>
+      <c r="B38" s="31" t="str">
         <f>B10</f>
         <v>-for brick wall</v>
       </c>
-      <c r="C38" s="35">
+      <c r="C38" s="32">
         <v>1</v>
       </c>
-      <c r="D38" s="36">
+      <c r="D38" s="33">
         <f>D10</f>
         <v>57.65</v>
       </c>
-      <c r="E38" s="36">
+      <c r="E38" s="33">
         <v>0.23</v>
       </c>
-      <c r="F38" s="36">
+      <c r="F38" s="33">
         <f>0.9+0.6-0.075*2</f>
         <v>1.35</v>
       </c>
-      <c r="G38" s="36">
+      <c r="G38" s="33">
         <f>PRODUCT(C38:F38)</f>
         <v>17.900325000000002</v>
       </c>
-      <c r="H38" s="21"/>
-      <c r="I38" s="21"/>
-      <c r="J38" s="21"/>
-      <c r="K38" s="21"/>
+      <c r="H38" s="20"/>
+      <c r="I38" s="20"/>
+      <c r="J38" s="20"/>
+      <c r="K38" s="20"/>
     </row>
     <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="9"/>
-      <c r="B39" s="10" t="s">
+      <c r="A39" s="8"/>
+      <c r="B39" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C39" s="11"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="14">
+      <c r="C39" s="10"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="13">
         <f>SUM(G38:G38)</f>
         <v>17.900325000000002</v>
       </c>
-      <c r="H39" s="15" t="s">
+      <c r="H39" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I39" s="14">
+      <c r="I39" s="13">
         <v>14491.84</v>
       </c>
-      <c r="J39" s="16">
+      <c r="J39" s="15">
         <f>G39*I39</f>
         <v>259408.64584800004</v>
       </c>
-      <c r="K39" s="13"/>
+      <c r="K39" s="12"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="33"/>
-      <c r="B40" s="37" t="s">
+      <c r="A40" s="30"/>
+      <c r="B40" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C40" s="21"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
-      <c r="G40" s="21"/>
-      <c r="H40" s="21"/>
-      <c r="I40" s="21"/>
-      <c r="J40" s="16">
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="15">
         <f>0.13*G39*10374.74</f>
         <v>24142.458312765004</v>
       </c>
-      <c r="K40" s="21"/>
+      <c r="K40" s="20"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" s="33"/>
-      <c r="B41" s="37"/>
-      <c r="C41" s="21"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
-      <c r="G41" s="21"/>
-      <c r="H41" s="21"/>
-      <c r="I41" s="21"/>
-      <c r="J41" s="16"/>
-      <c r="K41" s="21"/>
-    </row>
-    <row r="42" spans="1:11" s="17" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
-      <c r="A42" s="42">
+      <c r="A41" s="30"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
+      <c r="F41" s="20"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="20"/>
+      <c r="I41" s="20"/>
+      <c r="J41" s="15"/>
+      <c r="K41" s="20"/>
+    </row>
+    <row r="42" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+      <c r="A42" s="8">
         <v>6</v>
       </c>
-      <c r="B42" s="38" t="s">
+      <c r="B42" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="C42" s="44"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="45"/>
-      <c r="F42" s="45"/>
-      <c r="G42" s="46"/>
-      <c r="H42" s="47"/>
-      <c r="I42" s="14"/>
-      <c r="J42" s="46"/>
-      <c r="K42" s="45"/>
-    </row>
-    <row r="43" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="42"/>
-      <c r="B43" s="48" t="str">
+      <c r="C42" s="10"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="40"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="40"/>
+      <c r="K42" s="12"/>
+    </row>
+    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="8"/>
+      <c r="B43" s="41" t="str">
         <f>B28</f>
         <v>-for brick wall</v>
       </c>
-      <c r="C43" s="44">
+      <c r="C43" s="10">
         <v>2</v>
       </c>
-      <c r="D43" s="12">
+      <c r="D43" s="11">
         <f>D38+C11*D11</f>
         <v>65</v>
       </c>
-      <c r="E43" s="45"/>
-      <c r="F43" s="45">
+      <c r="E43" s="12"/>
+      <c r="F43" s="12">
         <v>0.9</v>
       </c>
-      <c r="G43" s="49">
+      <c r="G43" s="42">
         <f t="shared" ref="G43" si="1">PRODUCT(C43:F43)</f>
         <v>117</v>
       </c>
-      <c r="H43" s="47"/>
-      <c r="I43" s="14"/>
-      <c r="J43" s="46"/>
-      <c r="K43" s="45"/>
-    </row>
-    <row r="44" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="42"/>
-      <c r="B44" s="48" t="s">
+      <c r="H43" s="14"/>
+      <c r="I43" s="13"/>
+      <c r="J43" s="40"/>
+      <c r="K43" s="12"/>
+    </row>
+    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="8"/>
+      <c r="B44" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="C44" s="44"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="45"/>
-      <c r="F44" s="45"/>
-      <c r="G44" s="46">
+      <c r="C44" s="10"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="12"/>
+      <c r="F44" s="12"/>
+      <c r="G44" s="40">
         <f>SUM(G41:G43)</f>
         <v>117</v>
       </c>
-      <c r="H44" s="47" t="s">
+      <c r="H44" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="I44" s="14">
+      <c r="I44" s="13">
         <v>415.5</v>
       </c>
-      <c r="J44" s="46">
+      <c r="J44" s="40">
         <f>G44*I44</f>
         <v>48613.5</v>
       </c>
-      <c r="K44" s="45"/>
-    </row>
-    <row r="45" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="42"/>
-      <c r="B45" s="48" t="s">
+      <c r="K44" s="12"/>
+    </row>
+    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="8"/>
+      <c r="B45" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="C45" s="44"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="45"/>
-      <c r="G45" s="46"/>
-      <c r="H45" s="47"/>
-      <c r="I45" s="14"/>
-      <c r="J45" s="46">
+      <c r="C45" s="10"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="13"/>
+      <c r="J45" s="40">
         <f>0.13*G44*11650.4/100</f>
         <v>1772.02584</v>
       </c>
-      <c r="K45" s="45"/>
-    </row>
-    <row r="46" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="42"/>
-      <c r="B46" s="43"/>
-      <c r="C46" s="44"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="45"/>
-      <c r="F46" s="45"/>
-      <c r="G46" s="46"/>
-      <c r="H46" s="47"/>
-      <c r="I46" s="14"/>
-      <c r="J46" s="46"/>
-      <c r="K46" s="45"/>
-    </row>
-    <row r="47" spans="1:11" s="17" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
-      <c r="A47" s="42">
+      <c r="K45" s="12"/>
+    </row>
+    <row r="46" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="8"/>
+      <c r="B46" s="39"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="12"/>
+      <c r="G46" s="40"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="40"/>
+      <c r="K46" s="12"/>
+    </row>
+    <row r="47" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+      <c r="A47" s="8">
         <v>7</v>
       </c>
-      <c r="B47" s="38" t="s">
+      <c r="B47" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="C47" s="44"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="45"/>
-      <c r="F47" s="45"/>
-      <c r="G47" s="46"/>
-      <c r="H47" s="47"/>
-      <c r="I47" s="14"/>
-      <c r="J47" s="46"/>
-      <c r="K47" s="45"/>
-    </row>
-    <row r="48" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="42"/>
-      <c r="B48" s="48" t="str">
+      <c r="C47" s="10"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="40"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="13"/>
+      <c r="J47" s="40"/>
+      <c r="K47" s="12"/>
+    </row>
+    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="8"/>
+      <c r="B48" s="41" t="str">
         <f>B43</f>
         <v>-for brick wall</v>
       </c>
-      <c r="C48" s="44">
+      <c r="C48" s="10">
         <v>2</v>
       </c>
-      <c r="D48" s="12">
+      <c r="D48" s="11">
         <f>D43+C16*D16</f>
         <v>65</v>
       </c>
-      <c r="E48" s="45"/>
-      <c r="F48" s="45">
+      <c r="E48" s="12"/>
+      <c r="F48" s="12">
         <v>0.9</v>
       </c>
-      <c r="G48" s="49">
+      <c r="G48" s="42">
         <f t="shared" ref="G48" si="2">PRODUCT(C48:F48)</f>
         <v>117</v>
       </c>
-      <c r="H48" s="47"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="46"/>
-      <c r="K48" s="45"/>
-    </row>
-    <row r="49" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="42"/>
-      <c r="B49" s="48" t="s">
+      <c r="H48" s="14"/>
+      <c r="I48" s="13"/>
+      <c r="J48" s="40"/>
+      <c r="K48" s="12"/>
+    </row>
+    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="8"/>
+      <c r="B49" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="C49" s="44"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="45"/>
-      <c r="F49" s="45"/>
-      <c r="G49" s="46">
+      <c r="C49" s="10"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="12"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="40">
         <f>SUM(G46:G48)</f>
         <v>117</v>
       </c>
-      <c r="H49" s="47" t="s">
+      <c r="H49" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="I49" s="14">
+      <c r="I49" s="13">
         <v>253.8</v>
       </c>
-      <c r="J49" s="46">
+      <c r="J49" s="40">
         <f>G49*I49</f>
         <v>29694.600000000002</v>
       </c>
-      <c r="K49" s="45"/>
-    </row>
-    <row r="50" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="42"/>
-      <c r="B50" s="48" t="s">
+      <c r="K49" s="12"/>
+    </row>
+    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="8"/>
+      <c r="B50" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="C50" s="44"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="45"/>
-      <c r="F50" s="45"/>
-      <c r="G50" s="46"/>
-      <c r="H50" s="47"/>
-      <c r="I50" s="14"/>
-      <c r="J50" s="46">
+      <c r="C50" s="10"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="12"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="40"/>
+      <c r="H50" s="14"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="40">
         <f>0.13*G49*12736/100</f>
         <v>1937.1456000000001</v>
       </c>
-      <c r="K50" s="45"/>
-    </row>
-    <row r="51" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="42"/>
-      <c r="B51" s="43"/>
-      <c r="C51" s="44"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="45"/>
-      <c r="F51" s="45"/>
-      <c r="G51" s="46"/>
-      <c r="H51" s="47"/>
-      <c r="I51" s="14"/>
-      <c r="J51" s="46"/>
-      <c r="K51" s="45"/>
-    </row>
-    <row r="52" spans="1:11" s="8" customFormat="1" ht="90" x14ac:dyDescent="0.25">
-      <c r="A52" s="33">
+      <c r="K50" s="12"/>
+    </row>
+    <row r="51" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="8"/>
+      <c r="B51" s="39"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="12"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="40"/>
+      <c r="K51" s="12"/>
+    </row>
+    <row r="52" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A52" s="30">
         <v>8</v>
       </c>
       <c r="B52" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C52" s="32"/>
-      <c r="D52" s="32"/>
-      <c r="E52" s="32"/>
-      <c r="F52" s="32"/>
-      <c r="G52" s="32"/>
-      <c r="H52" s="32"/>
-      <c r="I52" s="32"/>
-      <c r="J52" s="32"/>
-      <c r="K52" s="32"/>
+      <c r="C52" s="20"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="20"/>
+      <c r="F52" s="20"/>
+      <c r="G52" s="20"/>
+      <c r="H52" s="20"/>
+      <c r="I52" s="20"/>
+      <c r="J52" s="20"/>
+      <c r="K52" s="20"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A53" s="33"/>
-      <c r="B53" s="34" t="str">
+      <c r="A53" s="30"/>
+      <c r="B53" s="31" t="str">
         <f>B12</f>
         <v>-for  stone masonary</v>
       </c>
-      <c r="C53" s="35">
+      <c r="C53" s="32">
         <v>1</v>
       </c>
-      <c r="D53" s="36">
+      <c r="D53" s="33">
         <f>D12</f>
         <v>58</v>
       </c>
-      <c r="E53" s="36">
+      <c r="E53" s="33">
         <f>((F53/2)+0.45)/2</f>
         <v>0.6</v>
       </c>
-      <c r="F53" s="36">
+      <c r="F53" s="33">
         <v>1.5</v>
       </c>
-      <c r="G53" s="36">
+      <c r="G53" s="33">
         <f>PRODUCT(C53:F53)</f>
         <v>52.199999999999996</v>
       </c>
-      <c r="H53" s="21"/>
-      <c r="I53" s="21"/>
-      <c r="J53" s="21"/>
-      <c r="K53" s="21"/>
+      <c r="H53" s="20"/>
+      <c r="I53" s="20"/>
+      <c r="J53" s="20"/>
+      <c r="K53" s="20"/>
     </row>
     <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="9"/>
-      <c r="B54" s="10" t="s">
+      <c r="A54" s="8"/>
+      <c r="B54" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C54" s="11"/>
-      <c r="D54" s="12"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="13"/>
-      <c r="G54" s="14">
+      <c r="C54" s="10"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="12"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="13">
         <f>SUM(G53:G53)</f>
         <v>52.199999999999996</v>
       </c>
-      <c r="H54" s="15" t="s">
+      <c r="H54" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="I54" s="14">
+      <c r="I54" s="13">
         <v>9878.43</v>
       </c>
-      <c r="J54" s="16">
+      <c r="J54" s="15">
         <f>G54*I54</f>
         <v>515654.04599999997</v>
       </c>
-      <c r="K54" s="13"/>
+      <c r="K54" s="12"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A55" s="33"/>
-      <c r="B55" s="37" t="s">
+      <c r="A55" s="30"/>
+      <c r="B55" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C55" s="21"/>
-      <c r="D55" s="21"/>
-      <c r="E55" s="21"/>
-      <c r="F55" s="21"/>
-      <c r="G55" s="21"/>
-      <c r="H55" s="21"/>
-      <c r="I55" s="21"/>
-      <c r="J55" s="16">
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="20"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="20"/>
+      <c r="H55" s="20"/>
+      <c r="I55" s="20"/>
+      <c r="J55" s="15">
         <f>0.13*G54*(27587.1)/5</f>
         <v>37441.212119999997</v>
       </c>
-      <c r="K55" s="21"/>
+      <c r="K55" s="20"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A56" s="33"/>
-      <c r="B56" s="21"/>
-      <c r="C56" s="21"/>
-      <c r="D56" s="21"/>
-      <c r="E56" s="21"/>
-      <c r="F56" s="21"/>
-      <c r="G56" s="21"/>
-      <c r="H56" s="21"/>
-      <c r="I56" s="21"/>
-      <c r="J56" s="21"/>
-      <c r="K56" s="21"/>
+      <c r="A56" s="30"/>
+      <c r="B56" s="20"/>
+      <c r="C56" s="20"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="20"/>
+      <c r="F56" s="20"/>
+      <c r="G56" s="20"/>
+      <c r="H56" s="20"/>
+      <c r="I56" s="20"/>
+      <c r="J56" s="20"/>
+      <c r="K56" s="20"/>
     </row>
     <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="9">
+      <c r="A57" s="8">
         <v>9</v>
       </c>
       <c r="B57" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C57" s="11">
+      <c r="C57" s="10">
         <v>1</v>
       </c>
-      <c r="D57" s="12"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="13"/>
-      <c r="G57" s="23">
+      <c r="D57" s="11"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="22">
         <f t="shared" ref="G57" si="3">PRODUCT(C57:F57)</f>
         <v>1</v>
       </c>
-      <c r="H57" s="15" t="s">
+      <c r="H57" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="I57" s="14">
+      <c r="I57" s="13">
         <v>500</v>
       </c>
-      <c r="J57" s="23">
+      <c r="J57" s="22">
         <f>G57*I57</f>
         <v>500</v>
       </c>
-      <c r="K57" s="13"/>
+      <c r="K57" s="12"/>
     </row>
     <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="9"/>
-      <c r="B58" s="22"/>
-      <c r="C58" s="11"/>
-      <c r="D58" s="12"/>
-      <c r="E58" s="13"/>
-      <c r="F58" s="13"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="15"/>
-      <c r="I58" s="14"/>
-      <c r="J58" s="16"/>
-      <c r="K58" s="13"/>
+      <c r="A58" s="8"/>
+      <c r="B58" s="21"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="12"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="14"/>
+      <c r="I58" s="13"/>
+      <c r="J58" s="15"/>
+      <c r="K58" s="12"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A59" s="20"/>
-      <c r="B59" s="30" t="s">
+      <c r="A59" s="19"/>
+      <c r="B59" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="C59" s="31"/>
-      <c r="D59" s="19"/>
-      <c r="E59" s="19"/>
-      <c r="F59" s="19"/>
-      <c r="G59" s="16"/>
-      <c r="H59" s="16"/>
-      <c r="I59" s="16"/>
-      <c r="J59" s="16">
+      <c r="C59" s="29"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="15"/>
+      <c r="H59" s="15"/>
+      <c r="I59" s="15"/>
+      <c r="J59" s="15">
         <f>SUM(J13:J57)</f>
         <v>1071666.46048649</v>
       </c>
-      <c r="K59" s="18"/>
-    </row>
-    <row r="61" spans="1:11" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="24"/>
-      <c r="B61" s="40" t="s">
+      <c r="K59" s="17"/>
+    </row>
+    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="23"/>
+      <c r="B61" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="C61" s="50">
+      <c r="C61" s="43">
         <f>J59</f>
         <v>1071666.46048649</v>
       </c>
-      <c r="D61" s="51"/>
-      <c r="E61" s="41">
+      <c r="D61" s="44"/>
+      <c r="E61" s="38">
         <v>100</v>
       </c>
-      <c r="F61" s="25"/>
-      <c r="G61" s="26"/>
-      <c r="H61" s="25"/>
-      <c r="I61" s="27"/>
-      <c r="J61" s="28"/>
-      <c r="K61" s="29"/>
+      <c r="F61" s="23"/>
+      <c r="G61" s="24"/>
+      <c r="H61" s="23"/>
+      <c r="I61" s="25"/>
+      <c r="J61" s="26"/>
+      <c r="K61" s="27"/>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B62" s="40" t="s">
+      <c r="B62" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="C62" s="56">
+      <c r="C62" s="49">
         <v>950000</v>
       </c>
-      <c r="D62" s="57"/>
-      <c r="E62" s="41"/>
+      <c r="D62" s="50"/>
+      <c r="E62" s="38"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B63" s="40" t="s">
+      <c r="B63" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="C63" s="56">
+      <c r="C63" s="49">
         <f>C62-C65-C66</f>
         <v>902500</v>
       </c>
-      <c r="D63" s="57"/>
-      <c r="E63" s="41">
+      <c r="D63" s="50"/>
+      <c r="E63" s="38">
         <f>C63/C61*100</f>
         <v>84.214635175790065</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B64" s="40" t="s">
+      <c r="B64" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="C64" s="62">
+      <c r="C64" s="55">
         <f>C61-C63</f>
         <v>169166.46048649005</v>
       </c>
-      <c r="D64" s="62"/>
-      <c r="E64" s="41">
+      <c r="D64" s="55"/>
+      <c r="E64" s="38">
         <f>100-E63</f>
         <v>15.785364824209935</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B65" s="40" t="s">
+      <c r="B65" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="C65" s="50">
+      <c r="C65" s="43">
         <f>C62*0.03</f>
         <v>28500</v>
       </c>
-      <c r="D65" s="51"/>
-      <c r="E65" s="41">
+      <c r="D65" s="44"/>
+      <c r="E65" s="38">
         <v>3</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B66" s="40" t="s">
+      <c r="B66" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="C66" s="50">
+      <c r="C66" s="43">
         <f>C62*0.02</f>
         <v>19000</v>
       </c>
-      <c r="D66" s="51"/>
-      <c r="E66" s="41">
+      <c r="D66" s="44"/>
+      <c r="E66" s="38">
         <v>2</v>
       </c>
     </row>
@@ -2356,4 +2311,1342 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3AD8C7E-C01D-4817-8DB8-B937A8E5E1AA}">
+  <dimension ref="A1:K66"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" customWidth="1"/>
+    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+    </row>
+    <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="46" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="47" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="47" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="47"/>
+    </row>
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="48" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="48"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+      <c r="K5" s="48"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="51" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="51"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="52" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="53" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="53"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="53"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="54"/>
+      <c r="J7" s="54"/>
+      <c r="K7" s="54"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+      <c r="A9" s="30">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="30"/>
+      <c r="B10" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="32">
+        <v>1</v>
+      </c>
+      <c r="D10" s="33">
+        <f>60-D11*C11</f>
+        <v>52.65</v>
+      </c>
+      <c r="E10" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="F10" s="33">
+        <v>0.75</v>
+      </c>
+      <c r="G10" s="33">
+        <f>PRODUCT(C10:F10)</f>
+        <v>11.846249999999998</v>
+      </c>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="20"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="30"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="32">
+        <v>21</v>
+      </c>
+      <c r="D11" s="33">
+        <v>0.35</v>
+      </c>
+      <c r="E11" s="33">
+        <v>0.35</v>
+      </c>
+      <c r="F11" s="33">
+        <v>1.75</v>
+      </c>
+      <c r="G11" s="33">
+        <f>PRODUCT(C11:F11)</f>
+        <v>4.5018750000000001</v>
+      </c>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="30"/>
+      <c r="B12" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="32">
+        <v>1</v>
+      </c>
+      <c r="D12" s="33">
+        <v>50</v>
+      </c>
+      <c r="E12" s="33">
+        <f>1.5/2</f>
+        <v>0.75</v>
+      </c>
+      <c r="F12" s="33">
+        <v>1.2</v>
+      </c>
+      <c r="G12" s="33">
+        <f>PRODUCT(C12:F12)</f>
+        <v>45</v>
+      </c>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+    </row>
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="13">
+        <f>SUM(G10:G12)</f>
+        <v>61.348124999999996</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I13" s="13">
+        <v>62.95</v>
+      </c>
+      <c r="J13" s="15">
+        <f>G13*I13</f>
+        <v>3861.86446875</v>
+      </c>
+      <c r="K13" s="12"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="30"/>
+      <c r="B14" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="15">
+        <f>0.13*G13*18612/360</f>
+        <v>412.32074812500002</v>
+      </c>
+      <c r="K14" s="20"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="30"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+    </row>
+    <row r="16" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A16" s="30">
+        <v>2</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="30"/>
+      <c r="B17" s="31" t="str">
+        <f>B12</f>
+        <v>-for  stone masonary</v>
+      </c>
+      <c r="C17" s="32">
+        <v>1</v>
+      </c>
+      <c r="D17" s="33">
+        <f>D12</f>
+        <v>50</v>
+      </c>
+      <c r="E17" s="33">
+        <f>1.5/2</f>
+        <v>0.75</v>
+      </c>
+      <c r="F17" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G17" s="33">
+        <f>PRODUCT(C17:F17)</f>
+        <v>5.625</v>
+      </c>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+    </row>
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="8"/>
+      <c r="B18" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="13">
+        <f>SUM(G17:G17)</f>
+        <v>5.625</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I18" s="13">
+        <v>4585.53</v>
+      </c>
+      <c r="J18" s="15">
+        <f>G18*I18</f>
+        <v>25793.606249999997</v>
+      </c>
+      <c r="K18" s="12"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="30"/>
+      <c r="B19" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="15">
+        <f>0.13*G18*15452.64/5</f>
+        <v>2259.9486000000002</v>
+      </c>
+      <c r="K19" s="20"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="30"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="20"/>
+    </row>
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="30">
+        <v>3</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="20"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="30"/>
+      <c r="B22" s="31" t="str">
+        <f>B10</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C22" s="32">
+        <v>1</v>
+      </c>
+      <c r="D22" s="33">
+        <f>D10</f>
+        <v>52.65</v>
+      </c>
+      <c r="E22" s="33">
+        <v>0.23</v>
+      </c>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33">
+        <f>PRODUCT(C22:F22)</f>
+        <v>12.109500000000001</v>
+      </c>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="30"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="32">
+        <f>C11</f>
+        <v>21</v>
+      </c>
+      <c r="D23" s="33">
+        <f>D11</f>
+        <v>0.35</v>
+      </c>
+      <c r="E23" s="33">
+        <f>E11</f>
+        <v>0.35</v>
+      </c>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33">
+        <f>PRODUCT(C23:F23)</f>
+        <v>2.5724999999999998</v>
+      </c>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
+    </row>
+    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="8"/>
+      <c r="B24" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="13">
+        <f>SUM(G22:G23)</f>
+        <v>14.682</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I24" s="13">
+        <v>1017.47</v>
+      </c>
+      <c r="J24" s="15">
+        <f>G24*I24</f>
+        <v>14938.494540000002</v>
+      </c>
+      <c r="K24" s="12"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="30"/>
+      <c r="B25" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="15">
+        <f>0.13*G24*8617.2/10</f>
+        <v>1644.7304952000002</v>
+      </c>
+      <c r="K25" s="20"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="30"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="20"/>
+    </row>
+    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A27" s="30">
+        <v>4</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
+      <c r="I27" s="20"/>
+      <c r="J27" s="20"/>
+      <c r="K27" s="20"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="30"/>
+      <c r="B28" s="31" t="str">
+        <f>B10</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C28" s="20">
+        <v>1</v>
+      </c>
+      <c r="D28" s="36">
+        <f>D10</f>
+        <v>52.65</v>
+      </c>
+      <c r="E28" s="20">
+        <v>0.23</v>
+      </c>
+      <c r="F28" s="33">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G28" s="33">
+        <f t="shared" ref="G28:G33" si="0">PRODUCT(C28:F28)</f>
+        <v>0.90821249999999998</v>
+      </c>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="30"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="20">
+        <v>2</v>
+      </c>
+      <c r="D29" s="36">
+        <f>D10</f>
+        <v>52.65</v>
+      </c>
+      <c r="E29" s="20">
+        <v>0.23</v>
+      </c>
+      <c r="F29" s="33">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G29" s="33">
+        <f t="shared" si="0"/>
+        <v>1.816425</v>
+      </c>
+      <c r="H29" s="20"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="20"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="30"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="20">
+        <f>C11</f>
+        <v>21</v>
+      </c>
+      <c r="D30" s="36">
+        <f>D11</f>
+        <v>0.35</v>
+      </c>
+      <c r="E30" s="36">
+        <f>E11</f>
+        <v>0.35</v>
+      </c>
+      <c r="F30" s="36">
+        <v>0.05</v>
+      </c>
+      <c r="G30" s="33">
+        <f t="shared" si="0"/>
+        <v>0.12862499999999999</v>
+      </c>
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="20"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="30"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="20">
+        <f>21*2</f>
+        <v>42</v>
+      </c>
+      <c r="D31" s="36">
+        <v>0.35</v>
+      </c>
+      <c r="E31" s="36">
+        <v>0.35</v>
+      </c>
+      <c r="F31" s="36">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G31" s="33">
+        <f t="shared" si="0"/>
+        <v>0.38587499999999997</v>
+      </c>
+      <c r="H31" s="20"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="30"/>
+      <c r="B32" s="31" t="str">
+        <f>B12</f>
+        <v>-for  stone masonary</v>
+      </c>
+      <c r="C32" s="32">
+        <v>1</v>
+      </c>
+      <c r="D32" s="33">
+        <f>D12</f>
+        <v>50</v>
+      </c>
+      <c r="E32" s="33">
+        <f>F53/2</f>
+        <v>0.6</v>
+      </c>
+      <c r="F32" s="33">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G32" s="33">
+        <f t="shared" si="0"/>
+        <v>2.25</v>
+      </c>
+      <c r="H32" s="20"/>
+      <c r="I32" s="20"/>
+      <c r="J32" s="20"/>
+      <c r="K32" s="20"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="30"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="32">
+        <v>1</v>
+      </c>
+      <c r="D33" s="33">
+        <f>D32</f>
+        <v>50</v>
+      </c>
+      <c r="E33" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="F33" s="33">
+        <v>0.05</v>
+      </c>
+      <c r="G33" s="33">
+        <f t="shared" si="0"/>
+        <v>1.125</v>
+      </c>
+      <c r="H33" s="20"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="20"/>
+      <c r="K33" s="20"/>
+    </row>
+    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="8"/>
+      <c r="B34" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="10"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="13">
+        <f>SUM(G28:G33)</f>
+        <v>6.6141375</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I34" s="13">
+        <v>10964.46</v>
+      </c>
+      <c r="J34" s="15">
+        <f>G34*I34</f>
+        <v>72520.446053249994</v>
+      </c>
+      <c r="K34" s="12"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="30"/>
+      <c r="B35" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="20"/>
+      <c r="I35" s="20"/>
+      <c r="J35" s="15">
+        <f>0.13*G34*(119450.3+6325.7)/15</f>
+        <v>7209.7979044000003</v>
+      </c>
+      <c r="K35" s="20"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="30"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="20"/>
+      <c r="I36" s="20"/>
+      <c r="J36" s="20"/>
+      <c r="K36" s="20"/>
+    </row>
+    <row r="37" spans="1:11" ht="32.25" x14ac:dyDescent="0.25">
+      <c r="A37" s="30">
+        <v>5</v>
+      </c>
+      <c r="B37" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="20"/>
+      <c r="I37" s="20"/>
+      <c r="J37" s="20"/>
+      <c r="K37" s="20"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="30"/>
+      <c r="B38" s="31" t="str">
+        <f>B10</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C38" s="32">
+        <v>1</v>
+      </c>
+      <c r="D38" s="33">
+        <f>D10</f>
+        <v>52.65</v>
+      </c>
+      <c r="E38" s="33">
+        <v>0.23</v>
+      </c>
+      <c r="F38" s="33">
+        <f>0.9+0.6-0.075*2</f>
+        <v>1.35</v>
+      </c>
+      <c r="G38" s="33">
+        <f>PRODUCT(C38:F38)</f>
+        <v>16.347825</v>
+      </c>
+      <c r="H38" s="20"/>
+      <c r="I38" s="20"/>
+      <c r="J38" s="20"/>
+      <c r="K38" s="20"/>
+    </row>
+    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="8"/>
+      <c r="B39" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="10"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="13">
+        <f>SUM(G38:G38)</f>
+        <v>16.347825</v>
+      </c>
+      <c r="H39" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I39" s="13">
+        <v>14491.84</v>
+      </c>
+      <c r="J39" s="15">
+        <f>G39*I39</f>
+        <v>236910.06424800001</v>
+      </c>
+      <c r="K39" s="12"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="30"/>
+      <c r="B40" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="15">
+        <f>0.13*G39*10374.74</f>
+        <v>22048.576412265</v>
+      </c>
+      <c r="K40" s="20"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="30"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
+      <c r="F41" s="20"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="20"/>
+      <c r="I41" s="20"/>
+      <c r="J41" s="15"/>
+      <c r="K41" s="20"/>
+    </row>
+    <row r="42" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+      <c r="A42" s="8">
+        <v>6</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C42" s="10"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="40"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="40"/>
+      <c r="K42" s="12"/>
+    </row>
+    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="8"/>
+      <c r="B43" s="41" t="str">
+        <f>B28</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C43" s="10">
+        <v>2</v>
+      </c>
+      <c r="D43" s="11">
+        <f>D38+C11*D11</f>
+        <v>60</v>
+      </c>
+      <c r="E43" s="12"/>
+      <c r="F43" s="12">
+        <v>0.9</v>
+      </c>
+      <c r="G43" s="42">
+        <f t="shared" ref="G43" si="1">PRODUCT(C43:F43)</f>
+        <v>108</v>
+      </c>
+      <c r="H43" s="14"/>
+      <c r="I43" s="13"/>
+      <c r="J43" s="40"/>
+      <c r="K43" s="12"/>
+    </row>
+    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="8"/>
+      <c r="B44" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="C44" s="10"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="12"/>
+      <c r="F44" s="12"/>
+      <c r="G44" s="40">
+        <f>SUM(G41:G43)</f>
+        <v>108</v>
+      </c>
+      <c r="H44" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="I44" s="13">
+        <v>415.5</v>
+      </c>
+      <c r="J44" s="40">
+        <f>G44*I44</f>
+        <v>44874</v>
+      </c>
+      <c r="K44" s="12"/>
+    </row>
+    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="8"/>
+      <c r="B45" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="C45" s="10"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="13"/>
+      <c r="J45" s="40">
+        <f>0.13*G44*11650.4/100</f>
+        <v>1635.7161600000002</v>
+      </c>
+      <c r="K45" s="12"/>
+    </row>
+    <row r="46" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="8"/>
+      <c r="B46" s="39"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="12"/>
+      <c r="G46" s="40"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="40"/>
+      <c r="K46" s="12"/>
+    </row>
+    <row r="47" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+      <c r="A47" s="8">
+        <v>7</v>
+      </c>
+      <c r="B47" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="C47" s="10"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="40"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="13"/>
+      <c r="J47" s="40"/>
+      <c r="K47" s="12"/>
+    </row>
+    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="8"/>
+      <c r="B48" s="41" t="str">
+        <f>B43</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C48" s="10">
+        <v>2</v>
+      </c>
+      <c r="D48" s="11">
+        <f>D43</f>
+        <v>60</v>
+      </c>
+      <c r="E48" s="12"/>
+      <c r="F48" s="12">
+        <v>0.9</v>
+      </c>
+      <c r="G48" s="42">
+        <f t="shared" ref="G48" si="2">PRODUCT(C48:F48)</f>
+        <v>108</v>
+      </c>
+      <c r="H48" s="14"/>
+      <c r="I48" s="13"/>
+      <c r="J48" s="40"/>
+      <c r="K48" s="12"/>
+    </row>
+    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="8"/>
+      <c r="B49" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="C49" s="10"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="12"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="40">
+        <f>SUM(G46:G48)</f>
+        <v>108</v>
+      </c>
+      <c r="H49" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="I49" s="13">
+        <v>253.8</v>
+      </c>
+      <c r="J49" s="40">
+        <f>G49*I49</f>
+        <v>27410.400000000001</v>
+      </c>
+      <c r="K49" s="12"/>
+    </row>
+    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="8"/>
+      <c r="B50" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" s="10"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="12"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="40"/>
+      <c r="H50" s="14"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="40">
+        <f>0.13*G49*12736/100</f>
+        <v>1788.1343999999999</v>
+      </c>
+      <c r="K50" s="12"/>
+    </row>
+    <row r="51" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="8"/>
+      <c r="B51" s="39"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="12"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="40"/>
+      <c r="K51" s="12"/>
+    </row>
+    <row r="52" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A52" s="30">
+        <v>8</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C52" s="20"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="20"/>
+      <c r="F52" s="20"/>
+      <c r="G52" s="20"/>
+      <c r="H52" s="20"/>
+      <c r="I52" s="20"/>
+      <c r="J52" s="20"/>
+      <c r="K52" s="20"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="30"/>
+      <c r="B53" s="31" t="str">
+        <f>B12</f>
+        <v>-for  stone masonary</v>
+      </c>
+      <c r="C53" s="32">
+        <v>1</v>
+      </c>
+      <c r="D53" s="33">
+        <f>D12</f>
+        <v>50</v>
+      </c>
+      <c r="E53" s="33">
+        <f>((F53/2)+0.45)/2</f>
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="F53" s="33">
+        <v>1.2</v>
+      </c>
+      <c r="G53" s="33">
+        <f>PRODUCT(C53:F53)</f>
+        <v>31.5</v>
+      </c>
+      <c r="H53" s="20"/>
+      <c r="I53" s="20"/>
+      <c r="J53" s="20"/>
+      <c r="K53" s="20"/>
+    </row>
+    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="8"/>
+      <c r="B54" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54" s="10"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="12"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="13">
+        <f>SUM(G53:G53)</f>
+        <v>31.5</v>
+      </c>
+      <c r="H54" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I54" s="13">
+        <v>9878.43</v>
+      </c>
+      <c r="J54" s="15">
+        <f>G54*I54</f>
+        <v>311170.54499999998</v>
+      </c>
+      <c r="K54" s="12"/>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="30"/>
+      <c r="B55" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="20"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="20"/>
+      <c r="H55" s="20"/>
+      <c r="I55" s="20"/>
+      <c r="J55" s="15">
+        <f>0.13*G54*(27587.1)/5</f>
+        <v>22593.834899999998</v>
+      </c>
+      <c r="K55" s="20"/>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="30"/>
+      <c r="B56" s="20"/>
+      <c r="C56" s="20"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="20"/>
+      <c r="F56" s="20"/>
+      <c r="G56" s="20"/>
+      <c r="H56" s="20"/>
+      <c r="I56" s="20"/>
+      <c r="J56" s="20"/>
+      <c r="K56" s="20"/>
+    </row>
+    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="8">
+        <v>9</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C57" s="10">
+        <v>1</v>
+      </c>
+      <c r="D57" s="11"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="22">
+        <f t="shared" ref="G57" si="3">PRODUCT(C57:F57)</f>
+        <v>1</v>
+      </c>
+      <c r="H57" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I57" s="13">
+        <v>500</v>
+      </c>
+      <c r="J57" s="22">
+        <f>G57*I57</f>
+        <v>500</v>
+      </c>
+      <c r="K57" s="12"/>
+    </row>
+    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="8"/>
+      <c r="B58" s="21"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="12"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="14"/>
+      <c r="I58" s="13"/>
+      <c r="J58" s="15"/>
+      <c r="K58" s="12"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="19"/>
+      <c r="B59" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C59" s="29"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="15"/>
+      <c r="H59" s="15"/>
+      <c r="I59" s="15"/>
+      <c r="J59" s="15">
+        <f>SUM(J13:J57)</f>
+        <v>797572.48017999006</v>
+      </c>
+      <c r="K59" s="17"/>
+    </row>
+    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="23"/>
+      <c r="B61" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="C61" s="43">
+        <f>J59</f>
+        <v>797572.48017999006</v>
+      </c>
+      <c r="D61" s="44"/>
+      <c r="E61" s="38">
+        <v>100</v>
+      </c>
+      <c r="F61" s="23"/>
+      <c r="G61" s="24"/>
+      <c r="H61" s="23"/>
+      <c r="I61" s="25"/>
+      <c r="J61" s="26"/>
+      <c r="K61" s="27"/>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B62" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="C62" s="49">
+        <v>500000</v>
+      </c>
+      <c r="D62" s="50"/>
+      <c r="E62" s="38"/>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B63" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="C63" s="49">
+        <f>C62-C65-C66</f>
+        <v>475000</v>
+      </c>
+      <c r="D63" s="50"/>
+      <c r="E63" s="38">
+        <f>C63/C61*100</f>
+        <v>59.555715850778299</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B64" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="C64" s="55">
+        <f>C61-C63</f>
+        <v>322572.48017999006</v>
+      </c>
+      <c r="D64" s="55"/>
+      <c r="E64" s="38">
+        <f>100-E63</f>
+        <v>40.444284149221701</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B65" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="C65" s="43">
+        <f>C62*0.03</f>
+        <v>15000</v>
+      </c>
+      <c r="D65" s="44"/>
+      <c r="E65" s="38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B66" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="C66" s="43">
+        <f>C62*0.02</f>
+        <v>10000</v>
+      </c>
+      <c r="D66" s="44"/>
+      <c r="E66" s="38">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
police chauki 500k pdf
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/police chauki.xlsx
+++ b/बजेट माग estimate/police chauki.xlsx
@@ -1,41 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18D42E1-AA93-40BB-AC38-5E32F4AE5403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040" firstSheet="2" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Estimate (4)" sheetId="10" state="hidden" r:id="rId1"/>
-    <sheet name="Police sector contribution" sheetId="11" r:id="rId2"/>
+    <sheet name="Police sector contribution" sheetId="11" state="hidden" r:id="rId2"/>
+    <sheet name="Police sector contribution (2)" sheetId="12" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
     <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <definedNames>
     <definedName name="description_103">[1]Abstract!$B$16</definedName>
     <definedName name="description_124" localSheetId="0">#REF!</definedName>
     <definedName name="description_124" localSheetId="1">#REF!</definedName>
+    <definedName name="description_124" localSheetId="2">#REF!</definedName>
     <definedName name="description_124">#REF!</definedName>
     <definedName name="description_247">[1]Abstract!$B$22</definedName>
     <definedName name="description_248">[1]Abstract!$B$23</definedName>
     <definedName name="description_261">[2]Abstract!$B$33</definedName>
     <definedName name="description_262">[1]Abstract!$B$34</definedName>
     <definedName name="description_3">[1]Abstract!$B$169</definedName>
+    <definedName name="description_310" localSheetId="2">#REF!</definedName>
     <definedName name="description_310">#REF!</definedName>
+    <definedName name="description_312" localSheetId="2">#REF!</definedName>
     <definedName name="description_312">#REF!</definedName>
     <definedName name="description_5">[1]Abstract!$B$171</definedName>
+    <definedName name="description_6" localSheetId="2">#REF!</definedName>
     <definedName name="description_6">#REF!</definedName>
     <definedName name="description_759">[1]Abstract!$B$278</definedName>
+    <definedName name="description_781" localSheetId="2">#REF!</definedName>
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Estimate (4)'!$A$5:$K$66</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Police sector contribution'!$A$5:$K$66</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Police sector contribution (2)'!$A$1:$K$66</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Police sector contribution (2)'!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -51,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="46">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -194,10 +201,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -372,21 +379,21 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -401,7 +408,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -439,7 +446,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -448,7 +455,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -538,7 +545,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -632,7 +639,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -691,9 +698,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -731,9 +738,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -768,7 +775,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -803,7 +810,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -976,22 +983,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K66"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="30.85546875" customWidth="1"/>
-    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
@@ -1006,7 +1013,7 @@
       <c r="J1" s="45"/>
       <c r="K1" s="45"/>
     </row>
-    <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A2" s="46" t="s">
         <v>1</v>
       </c>
@@ -1021,7 +1028,7 @@
       <c r="J2" s="46"/>
       <c r="K2" s="46"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="47" t="s">
         <v>2</v>
       </c>
@@ -1036,7 +1043,7 @@
       <c r="J3" s="47"/>
       <c r="K3" s="47"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="47" t="s">
         <v>3</v>
       </c>
@@ -1051,7 +1058,7 @@
       <c r="J4" s="47"/>
       <c r="K4" s="47"/>
     </row>
-    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A5" s="48" t="s">
         <v>4</v>
       </c>
@@ -1066,7 +1073,7 @@
       <c r="J5" s="48"/>
       <c r="K5" s="48"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="51" t="s">
         <v>42</v>
       </c>
@@ -1083,7 +1090,7 @@
       <c r="J6" s="52"/>
       <c r="K6" s="52"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="53" t="s">
         <v>5</v>
       </c>
@@ -1100,7 +1107,7 @@
       <c r="J7" s="54"/>
       <c r="K7" s="54"/>
     </row>
-    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -1135,7 +1142,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A9" s="30">
         <v>1</v>
       </c>
@@ -1152,7 +1159,7 @@
       <c r="J9" s="20"/>
       <c r="K9" s="20"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="30"/>
       <c r="B10" s="31" t="s">
         <v>25</v>
@@ -1179,7 +1186,7 @@
       <c r="J10" s="20"/>
       <c r="K10" s="20"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="30"/>
       <c r="B11" s="31"/>
       <c r="C11" s="32">
@@ -1203,7 +1210,7 @@
       <c r="J11" s="20"/>
       <c r="K11" s="20"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="30"/>
       <c r="B12" s="31" t="s">
         <v>26</v>
@@ -1230,7 +1237,7 @@
       <c r="J12" s="20"/>
       <c r="K12" s="20"/>
     </row>
-    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8"/>
       <c r="B13" s="9" t="s">
         <v>18</v>
@@ -1255,7 +1262,7 @@
       </c>
       <c r="K13" s="12"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="30"/>
       <c r="B14" s="34" t="s">
         <v>27</v>
@@ -1273,7 +1280,7 @@
       </c>
       <c r="K14" s="20"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="30"/>
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
@@ -1286,7 +1293,7 @@
       <c r="J15" s="20"/>
       <c r="K15" s="20"/>
     </row>
-    <row r="16" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A16" s="30">
         <v>2</v>
       </c>
@@ -1303,7 +1310,7 @@
       <c r="J16" s="20"/>
       <c r="K16" s="20"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="30"/>
       <c r="B17" s="31" t="str">
         <f>B12</f>
@@ -1332,7 +1339,7 @@
       <c r="J17" s="20"/>
       <c r="K17" s="20"/>
     </row>
-    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8"/>
       <c r="B18" s="9" t="s">
         <v>18</v>
@@ -1357,7 +1364,7 @@
       </c>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="30"/>
       <c r="B19" s="34" t="s">
         <v>27</v>
@@ -1375,7 +1382,7 @@
       </c>
       <c r="K19" s="20"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="30"/>
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
@@ -1388,7 +1395,7 @@
       <c r="J20" s="20"/>
       <c r="K20" s="20"/>
     </row>
-    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A21" s="30">
         <v>3</v>
       </c>
@@ -1405,7 +1412,7 @@
       <c r="J21" s="20"/>
       <c r="K21" s="20"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="30"/>
       <c r="B22" s="31" t="str">
         <f>B10</f>
@@ -1431,7 +1438,7 @@
       <c r="J22" s="20"/>
       <c r="K22" s="20"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="30"/>
       <c r="B23" s="31"/>
       <c r="C23" s="32">
@@ -1456,7 +1463,7 @@
       <c r="J23" s="20"/>
       <c r="K23" s="20"/>
     </row>
-    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
       <c r="B24" s="9" t="s">
         <v>18</v>
@@ -1481,7 +1488,7 @@
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="30"/>
       <c r="B25" s="34" t="s">
         <v>27</v>
@@ -1499,7 +1506,7 @@
       </c>
       <c r="K25" s="20"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="30"/>
       <c r="B26" s="20"/>
       <c r="C26" s="20"/>
@@ -1512,7 +1519,7 @@
       <c r="J26" s="20"/>
       <c r="K26" s="20"/>
     </row>
-    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="69" x14ac:dyDescent="0.3">
       <c r="A27" s="30">
         <v>4</v>
       </c>
@@ -1529,7 +1536,7 @@
       <c r="J27" s="20"/>
       <c r="K27" s="20"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="30"/>
       <c r="B28" s="31" t="str">
         <f>B10</f>
@@ -1557,7 +1564,7 @@
       <c r="J28" s="20"/>
       <c r="K28" s="20"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="30"/>
       <c r="B29" s="31"/>
       <c r="C29" s="20">
@@ -1582,7 +1589,7 @@
       <c r="J29" s="20"/>
       <c r="K29" s="20"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="30"/>
       <c r="B30" s="31"/>
       <c r="C30" s="20">
@@ -1609,7 +1616,7 @@
       <c r="J30" s="20"/>
       <c r="K30" s="20"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="30"/>
       <c r="B31" s="31"/>
       <c r="C31" s="20">
@@ -1634,7 +1641,7 @@
       <c r="J31" s="20"/>
       <c r="K31" s="20"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="30"/>
       <c r="B32" s="31" t="str">
         <f>B12</f>
@@ -1663,7 +1670,7 @@
       <c r="J32" s="20"/>
       <c r="K32" s="20"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="30"/>
       <c r="B33" s="31"/>
       <c r="C33" s="32">
@@ -1688,7 +1695,7 @@
       <c r="J33" s="20"/>
       <c r="K33" s="20"/>
     </row>
-    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="8"/>
       <c r="B34" s="9" t="s">
         <v>18</v>
@@ -1713,7 +1720,7 @@
       </c>
       <c r="K34" s="12"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="30"/>
       <c r="B35" s="34" t="s">
         <v>27</v>
@@ -1731,7 +1738,7 @@
       </c>
       <c r="K35" s="20"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="30"/>
       <c r="B36" s="20"/>
       <c r="C36" s="20"/>
@@ -1744,7 +1751,7 @@
       <c r="J36" s="20"/>
       <c r="K36" s="20"/>
     </row>
-    <row r="37" spans="1:11" ht="32.25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="33" x14ac:dyDescent="0.3">
       <c r="A37" s="30">
         <v>5</v>
       </c>
@@ -1761,7 +1768,7 @@
       <c r="J37" s="20"/>
       <c r="K37" s="20"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="30"/>
       <c r="B38" s="31" t="str">
         <f>B10</f>
@@ -1790,7 +1797,7 @@
       <c r="J38" s="20"/>
       <c r="K38" s="20"/>
     </row>
-    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="8"/>
       <c r="B39" s="9" t="s">
         <v>18</v>
@@ -1815,7 +1822,7 @@
       </c>
       <c r="K39" s="12"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="30"/>
       <c r="B40" s="34" t="s">
         <v>27</v>
@@ -1833,7 +1840,7 @@
       </c>
       <c r="K40" s="20"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="30"/>
       <c r="B41" s="34"/>
       <c r="C41" s="20"/>
@@ -1846,7 +1853,7 @@
       <c r="J41" s="15"/>
       <c r="K41" s="20"/>
     </row>
-    <row r="42" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
         <v>6</v>
       </c>
@@ -1863,7 +1870,7 @@
       <c r="J42" s="40"/>
       <c r="K42" s="12"/>
     </row>
-    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="8"/>
       <c r="B43" s="41" t="str">
         <f>B28</f>
@@ -1889,7 +1896,7 @@
       <c r="J43" s="40"/>
       <c r="K43" s="12"/>
     </row>
-    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="8"/>
       <c r="B44" s="41" t="s">
         <v>38</v>
@@ -1914,7 +1921,7 @@
       </c>
       <c r="K44" s="12"/>
     </row>
-    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
       <c r="B45" s="41" t="s">
         <v>40</v>
@@ -1932,7 +1939,7 @@
       </c>
       <c r="K45" s="12"/>
     </row>
-    <row r="46" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
       <c r="A46" s="8"/>
       <c r="B46" s="39"/>
       <c r="C46" s="10"/>
@@ -1945,7 +1952,7 @@
       <c r="J46" s="40"/>
       <c r="K46" s="12"/>
     </row>
-    <row r="47" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
         <v>7</v>
       </c>
@@ -1962,7 +1969,7 @@
       <c r="J47" s="40"/>
       <c r="K47" s="12"/>
     </row>
-    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
       <c r="B48" s="41" t="str">
         <f>B43</f>
@@ -1988,7 +1995,7 @@
       <c r="J48" s="40"/>
       <c r="K48" s="12"/>
     </row>
-    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="8"/>
       <c r="B49" s="41" t="s">
         <v>38</v>
@@ -2013,7 +2020,7 @@
       </c>
       <c r="K49" s="12"/>
     </row>
-    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="8"/>
       <c r="B50" s="41" t="s">
         <v>40</v>
@@ -2031,7 +2038,7 @@
       </c>
       <c r="K50" s="12"/>
     </row>
-    <row r="51" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
       <c r="A51" s="8"/>
       <c r="B51" s="39"/>
       <c r="C51" s="10"/>
@@ -2044,7 +2051,7 @@
       <c r="J51" s="40"/>
       <c r="K51" s="12"/>
     </row>
-    <row r="52" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A52" s="30">
         <v>8</v>
       </c>
@@ -2061,7 +2068,7 @@
       <c r="J52" s="20"/>
       <c r="K52" s="20"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" s="30"/>
       <c r="B53" s="31" t="str">
         <f>B12</f>
@@ -2090,7 +2097,7 @@
       <c r="J53" s="20"/>
       <c r="K53" s="20"/>
     </row>
-    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="8"/>
       <c r="B54" s="9" t="s">
         <v>18</v>
@@ -2115,7 +2122,7 @@
       </c>
       <c r="K54" s="12"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="30"/>
       <c r="B55" s="34" t="s">
         <v>27</v>
@@ -2133,7 +2140,7 @@
       </c>
       <c r="K55" s="20"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" s="30"/>
       <c r="B56" s="20"/>
       <c r="C56" s="20"/>
@@ -2146,7 +2153,7 @@
       <c r="J56" s="20"/>
       <c r="K56" s="20"/>
     </row>
-    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="8">
         <v>9</v>
       </c>
@@ -2175,7 +2182,7 @@
       </c>
       <c r="K57" s="12"/>
     </row>
-    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="8"/>
       <c r="B58" s="21"/>
       <c r="C58" s="10"/>
@@ -2188,7 +2195,7 @@
       <c r="J58" s="15"/>
       <c r="K58" s="12"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="19"/>
       <c r="B59" s="28" t="s">
         <v>23</v>
@@ -2206,7 +2213,7 @@
       </c>
       <c r="K59" s="17"/>
     </row>
-    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="23"/>
       <c r="B61" s="37" t="s">
         <v>22</v>
@@ -2226,7 +2233,7 @@
       <c r="J61" s="26"/>
       <c r="K61" s="27"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B62" s="37" t="s">
         <v>33</v>
       </c>
@@ -2236,7 +2243,7 @@
       <c r="D62" s="50"/>
       <c r="E62" s="38"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B63" s="37" t="s">
         <v>34</v>
       </c>
@@ -2250,7 +2257,7 @@
         <v>84.214635175790065</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B64" s="37" t="s">
         <v>32</v>
       </c>
@@ -2264,7 +2271,7 @@
         <v>15.785364824209935</v>
       </c>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B65" s="37" t="s">
         <v>35</v>
       </c>
@@ -2277,7 +2284,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B66" s="37" t="s">
         <v>36</v>
       </c>
@@ -2314,22 +2321,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3AD8C7E-C01D-4817-8DB8-B937A8E5E1AA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K66"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="30.85546875" customWidth="1"/>
-    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
@@ -2344,7 +2351,7 @@
       <c r="J1" s="45"/>
       <c r="K1" s="45"/>
     </row>
-    <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A2" s="46" t="s">
         <v>1</v>
       </c>
@@ -2359,7 +2366,7 @@
       <c r="J2" s="46"/>
       <c r="K2" s="46"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="47" t="s">
         <v>2</v>
       </c>
@@ -2374,7 +2381,7 @@
       <c r="J3" s="47"/>
       <c r="K3" s="47"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="47" t="s">
         <v>3</v>
       </c>
@@ -2389,7 +2396,7 @@
       <c r="J4" s="47"/>
       <c r="K4" s="47"/>
     </row>
-    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A5" s="48" t="s">
         <v>4</v>
       </c>
@@ -2404,7 +2411,7 @@
       <c r="J5" s="48"/>
       <c r="K5" s="48"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="51" t="s">
         <v>42</v>
       </c>
@@ -2421,7 +2428,7 @@
       <c r="J6" s="52"/>
       <c r="K6" s="52"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="53" t="s">
         <v>5</v>
       </c>
@@ -2438,7 +2445,7 @@
       <c r="J7" s="54"/>
       <c r="K7" s="54"/>
     </row>
-    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -2473,7 +2480,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
       <c r="A9" s="30">
         <v>1</v>
       </c>
@@ -2490,7 +2497,7 @@
       <c r="J9" s="20"/>
       <c r="K9" s="20"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="30"/>
       <c r="B10" s="31" t="s">
         <v>25</v>
@@ -2517,7 +2524,7 @@
       <c r="J10" s="20"/>
       <c r="K10" s="20"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="30"/>
       <c r="B11" s="31"/>
       <c r="C11" s="32">
@@ -2541,7 +2548,7 @@
       <c r="J11" s="20"/>
       <c r="K11" s="20"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="30"/>
       <c r="B12" s="31" t="s">
         <v>26</v>
@@ -2568,7 +2575,7 @@
       <c r="J12" s="20"/>
       <c r="K12" s="20"/>
     </row>
-    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8"/>
       <c r="B13" s="9" t="s">
         <v>18</v>
@@ -2593,7 +2600,7 @@
       </c>
       <c r="K13" s="12"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="30"/>
       <c r="B14" s="34" t="s">
         <v>27</v>
@@ -2611,7 +2618,7 @@
       </c>
       <c r="K14" s="20"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="30"/>
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
@@ -2624,7 +2631,7 @@
       <c r="J15" s="20"/>
       <c r="K15" s="20"/>
     </row>
-    <row r="16" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A16" s="30">
         <v>2</v>
       </c>
@@ -2641,7 +2648,7 @@
       <c r="J16" s="20"/>
       <c r="K16" s="20"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="30"/>
       <c r="B17" s="31" t="str">
         <f>B12</f>
@@ -2670,7 +2677,7 @@
       <c r="J17" s="20"/>
       <c r="K17" s="20"/>
     </row>
-    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8"/>
       <c r="B18" s="9" t="s">
         <v>18</v>
@@ -2695,7 +2702,7 @@
       </c>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="30"/>
       <c r="B19" s="34" t="s">
         <v>27</v>
@@ -2713,7 +2720,7 @@
       </c>
       <c r="K19" s="20"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="30"/>
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
@@ -2726,7 +2733,7 @@
       <c r="J20" s="20"/>
       <c r="K20" s="20"/>
     </row>
-    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A21" s="30">
         <v>3</v>
       </c>
@@ -2743,7 +2750,7 @@
       <c r="J21" s="20"/>
       <c r="K21" s="20"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="30"/>
       <c r="B22" s="31" t="str">
         <f>B10</f>
@@ -2769,7 +2776,7 @@
       <c r="J22" s="20"/>
       <c r="K22" s="20"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="30"/>
       <c r="B23" s="31"/>
       <c r="C23" s="32">
@@ -2794,7 +2801,7 @@
       <c r="J23" s="20"/>
       <c r="K23" s="20"/>
     </row>
-    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
       <c r="B24" s="9" t="s">
         <v>18</v>
@@ -2819,7 +2826,7 @@
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="30"/>
       <c r="B25" s="34" t="s">
         <v>27</v>
@@ -2837,7 +2844,7 @@
       </c>
       <c r="K25" s="20"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="30"/>
       <c r="B26" s="20"/>
       <c r="C26" s="20"/>
@@ -2850,7 +2857,7 @@
       <c r="J26" s="20"/>
       <c r="K26" s="20"/>
     </row>
-    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="69" x14ac:dyDescent="0.3">
       <c r="A27" s="30">
         <v>4</v>
       </c>
@@ -2867,7 +2874,7 @@
       <c r="J27" s="20"/>
       <c r="K27" s="20"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="30"/>
       <c r="B28" s="31" t="str">
         <f>B10</f>
@@ -2895,7 +2902,7 @@
       <c r="J28" s="20"/>
       <c r="K28" s="20"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="30"/>
       <c r="B29" s="31"/>
       <c r="C29" s="20">
@@ -2920,7 +2927,7 @@
       <c r="J29" s="20"/>
       <c r="K29" s="20"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="30"/>
       <c r="B30" s="31"/>
       <c r="C30" s="20">
@@ -2947,7 +2954,7 @@
       <c r="J30" s="20"/>
       <c r="K30" s="20"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="30"/>
       <c r="B31" s="31"/>
       <c r="C31" s="20">
@@ -2972,7 +2979,7 @@
       <c r="J31" s="20"/>
       <c r="K31" s="20"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="30"/>
       <c r="B32" s="31" t="str">
         <f>B12</f>
@@ -3001,7 +3008,7 @@
       <c r="J32" s="20"/>
       <c r="K32" s="20"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="30"/>
       <c r="B33" s="31"/>
       <c r="C33" s="32">
@@ -3026,7 +3033,7 @@
       <c r="J33" s="20"/>
       <c r="K33" s="20"/>
     </row>
-    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="8"/>
       <c r="B34" s="9" t="s">
         <v>18</v>
@@ -3051,7 +3058,7 @@
       </c>
       <c r="K34" s="12"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="30"/>
       <c r="B35" s="34" t="s">
         <v>27</v>
@@ -3069,7 +3076,7 @@
       </c>
       <c r="K35" s="20"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="30"/>
       <c r="B36" s="20"/>
       <c r="C36" s="20"/>
@@ -3082,7 +3089,7 @@
       <c r="J36" s="20"/>
       <c r="K36" s="20"/>
     </row>
-    <row r="37" spans="1:11" ht="32.25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="33" x14ac:dyDescent="0.3">
       <c r="A37" s="30">
         <v>5</v>
       </c>
@@ -3099,7 +3106,7 @@
       <c r="J37" s="20"/>
       <c r="K37" s="20"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="30"/>
       <c r="B38" s="31" t="str">
         <f>B10</f>
@@ -3128,7 +3135,7 @@
       <c r="J38" s="20"/>
       <c r="K38" s="20"/>
     </row>
-    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="8"/>
       <c r="B39" s="9" t="s">
         <v>18</v>
@@ -3153,7 +3160,7 @@
       </c>
       <c r="K39" s="12"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="30"/>
       <c r="B40" s="34" t="s">
         <v>27</v>
@@ -3171,7 +3178,7 @@
       </c>
       <c r="K40" s="20"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="30"/>
       <c r="B41" s="34"/>
       <c r="C41" s="20"/>
@@ -3184,7 +3191,7 @@
       <c r="J41" s="15"/>
       <c r="K41" s="20"/>
     </row>
-    <row r="42" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
       <c r="A42" s="8">
         <v>6</v>
       </c>
@@ -3201,7 +3208,7 @@
       <c r="J42" s="40"/>
       <c r="K42" s="12"/>
     </row>
-    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="8"/>
       <c r="B43" s="41" t="str">
         <f>B28</f>
@@ -3227,7 +3234,7 @@
       <c r="J43" s="40"/>
       <c r="K43" s="12"/>
     </row>
-    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="8"/>
       <c r="B44" s="41" t="s">
         <v>38</v>
@@ -3252,7 +3259,7 @@
       </c>
       <c r="K44" s="12"/>
     </row>
-    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
       <c r="B45" s="41" t="s">
         <v>40</v>
@@ -3270,7 +3277,7 @@
       </c>
       <c r="K45" s="12"/>
     </row>
-    <row r="46" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
       <c r="A46" s="8"/>
       <c r="B46" s="39"/>
       <c r="C46" s="10"/>
@@ -3283,7 +3290,7 @@
       <c r="J46" s="40"/>
       <c r="K46" s="12"/>
     </row>
-    <row r="47" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
       <c r="A47" s="8">
         <v>7</v>
       </c>
@@ -3300,7 +3307,7 @@
       <c r="J47" s="40"/>
       <c r="K47" s="12"/>
     </row>
-    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
       <c r="B48" s="41" t="str">
         <f>B43</f>
@@ -3326,7 +3333,7 @@
       <c r="J48" s="40"/>
       <c r="K48" s="12"/>
     </row>
-    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="8"/>
       <c r="B49" s="41" t="s">
         <v>38</v>
@@ -3351,7 +3358,7 @@
       </c>
       <c r="K49" s="12"/>
     </row>
-    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="8"/>
       <c r="B50" s="41" t="s">
         <v>40</v>
@@ -3369,7 +3376,7 @@
       </c>
       <c r="K50" s="12"/>
     </row>
-    <row r="51" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
       <c r="A51" s="8"/>
       <c r="B51" s="39"/>
       <c r="C51" s="10"/>
@@ -3382,7 +3389,7 @@
       <c r="J51" s="40"/>
       <c r="K51" s="12"/>
     </row>
-    <row r="52" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A52" s="30">
         <v>8</v>
       </c>
@@ -3399,7 +3406,7 @@
       <c r="J52" s="20"/>
       <c r="K52" s="20"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" s="30"/>
       <c r="B53" s="31" t="str">
         <f>B12</f>
@@ -3428,7 +3435,7 @@
       <c r="J53" s="20"/>
       <c r="K53" s="20"/>
     </row>
-    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="8"/>
       <c r="B54" s="9" t="s">
         <v>18</v>
@@ -3453,7 +3460,7 @@
       </c>
       <c r="K54" s="12"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="30"/>
       <c r="B55" s="34" t="s">
         <v>27</v>
@@ -3471,7 +3478,7 @@
       </c>
       <c r="K55" s="20"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" s="30"/>
       <c r="B56" s="20"/>
       <c r="C56" s="20"/>
@@ -3484,7 +3491,7 @@
       <c r="J56" s="20"/>
       <c r="K56" s="20"/>
     </row>
-    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="8">
         <v>9</v>
       </c>
@@ -3513,7 +3520,7 @@
       </c>
       <c r="K57" s="12"/>
     </row>
-    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="8"/>
       <c r="B58" s="21"/>
       <c r="C58" s="10"/>
@@ -3526,7 +3533,7 @@
       <c r="J58" s="15"/>
       <c r="K58" s="12"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="19"/>
       <c r="B59" s="28" t="s">
         <v>23</v>
@@ -3544,7 +3551,7 @@
       </c>
       <c r="K59" s="17"/>
     </row>
-    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="23"/>
       <c r="B61" s="37" t="s">
         <v>22</v>
@@ -3564,7 +3571,7 @@
       <c r="J61" s="26"/>
       <c r="K61" s="27"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B62" s="37" t="s">
         <v>33</v>
       </c>
@@ -3574,7 +3581,7 @@
       <c r="D62" s="50"/>
       <c r="E62" s="38"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B63" s="37" t="s">
         <v>34</v>
       </c>
@@ -3588,7 +3595,7 @@
         <v>59.555715850778299</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B64" s="37" t="s">
         <v>45</v>
       </c>
@@ -3602,7 +3609,7 @@
         <v>40.444284149221701</v>
       </c>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B65" s="37" t="s">
         <v>35</v>
       </c>
@@ -3615,7 +3622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B66" s="37" t="s">
         <v>36</v>
       </c>
@@ -3638,15 +3645,1374 @@
     <mergeCell ref="C62:D62"/>
     <mergeCell ref="C63:D63"/>
     <mergeCell ref="C64:D64"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Q66"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" customWidth="1"/>
+    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+    </row>
+    <row r="2" spans="1:17" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="46" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
+      <c r="K2" s="46"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" s="47" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="47" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="47"/>
+    </row>
+    <row r="5" spans="1:17" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A5" s="48" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="48"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+      <c r="K5" s="48"/>
+    </row>
+    <row r="6" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="51" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="51"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="52" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
+      <c r="K6" s="52"/>
+    </row>
+    <row r="7" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="53" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="53"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="53"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="54"/>
+      <c r="J7" s="54"/>
+      <c r="K7" s="54"/>
+    </row>
+    <row r="8" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="124.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="30">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" s="30"/>
+      <c r="B10" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="32">
+        <v>1</v>
+      </c>
+      <c r="D10" s="33">
+        <f>45-D11*C11</f>
+        <v>39.4</v>
+      </c>
+      <c r="E10" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="F10" s="33">
+        <v>0.75</v>
+      </c>
+      <c r="G10" s="33">
+        <f>PRODUCT(C10:F10)</f>
+        <v>8.8649999999999984</v>
+      </c>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="20"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11" s="30"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="32">
+        <f>TRUNC(D17/3,0)+1</f>
+        <v>16</v>
+      </c>
+      <c r="D11" s="33">
+        <v>0.35</v>
+      </c>
+      <c r="E11" s="33">
+        <v>0.35</v>
+      </c>
+      <c r="F11" s="33">
+        <f>F10</f>
+        <v>0.75</v>
+      </c>
+      <c r="G11" s="33">
+        <f>PRODUCT(C11:F11)</f>
+        <v>1.4699999999999998</v>
+      </c>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+      <c r="O11">
+        <f>60/2.5</f>
+        <v>24</v>
+      </c>
+      <c r="P11">
+        <f>60/3</f>
+        <v>20</v>
+      </c>
+      <c r="Q11">
+        <f>50/3</f>
+        <v>16.666666666666668</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A12" s="30"/>
+      <c r="B12" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="32">
+        <v>1</v>
+      </c>
+      <c r="D12" s="33">
+        <v>45</v>
+      </c>
+      <c r="E12" s="33">
+        <f>1.5/2</f>
+        <v>0.75</v>
+      </c>
+      <c r="F12" s="33">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G12" s="33">
+        <f>PRODUCT(C12:F12)</f>
+        <v>33.75</v>
+      </c>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+    </row>
+    <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="8"/>
+      <c r="B13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="13">
+        <f>SUM(G10:G12)</f>
+        <v>44.084999999999994</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I13" s="13">
+        <v>62.95</v>
+      </c>
+      <c r="J13" s="15">
+        <f>G13*I13</f>
+        <v>2775.1507499999998</v>
+      </c>
+      <c r="K13" s="12"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A14" s="30"/>
+      <c r="B14" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="15">
+        <f>0.13*G13*18612/360</f>
+        <v>296.29528499999998</v>
+      </c>
+      <c r="K14" s="20"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A15" s="30"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+    </row>
+    <row r="16" spans="1:17" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="30">
+        <v>2</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="20"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="30"/>
+      <c r="B17" s="31" t="str">
+        <f>B12</f>
+        <v>-for  stone masonary</v>
+      </c>
+      <c r="C17" s="32">
+        <v>1</v>
+      </c>
+      <c r="D17" s="33">
+        <f>D12</f>
+        <v>45</v>
+      </c>
+      <c r="E17" s="33">
+        <f>1.5/2</f>
+        <v>0.75</v>
+      </c>
+      <c r="F17" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G17" s="33">
+        <f>PRODUCT(C17:F17)</f>
+        <v>5.0625</v>
+      </c>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+    </row>
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="8"/>
+      <c r="B18" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="13">
+        <f>SUM(G17:G17)</f>
+        <v>5.0625</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I18" s="13">
+        <v>4585.53</v>
+      </c>
+      <c r="J18" s="15">
+        <f>G18*I18</f>
+        <v>23214.245625</v>
+      </c>
+      <c r="K18" s="12"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="30"/>
+      <c r="B19" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="15">
+        <f>0.13*G18*15452.64/5</f>
+        <v>2033.9537400000002</v>
+      </c>
+      <c r="K19" s="20"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="30"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="20"/>
+    </row>
+    <row r="21" spans="1:11" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="30">
+        <v>3</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="20"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="30"/>
+      <c r="B22" s="31" t="str">
+        <f>B10</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C22" s="32">
+        <v>1</v>
+      </c>
+      <c r="D22" s="33">
+        <f>D10</f>
+        <v>39.4</v>
+      </c>
+      <c r="E22" s="33">
+        <v>0.23</v>
+      </c>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33">
+        <f>PRODUCT(C22:F22)</f>
+        <v>9.0619999999999994</v>
+      </c>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="30"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="32">
+        <f>C11</f>
+        <v>16</v>
+      </c>
+      <c r="D23" s="33">
+        <f>D11</f>
+        <v>0.35</v>
+      </c>
+      <c r="E23" s="33">
+        <f>E11</f>
+        <v>0.35</v>
+      </c>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33">
+        <f>PRODUCT(C23:F23)</f>
+        <v>1.9599999999999997</v>
+      </c>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
+    </row>
+    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="8"/>
+      <c r="B24" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="13">
+        <f>SUM(G22:G23)</f>
+        <v>11.021999999999998</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I24" s="13">
+        <v>1017.47</v>
+      </c>
+      <c r="J24" s="15">
+        <f>G24*I24</f>
+        <v>11214.554339999999</v>
+      </c>
+      <c r="K24" s="12"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" s="30"/>
+      <c r="B25" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="15">
+        <f>0.13*G24*8617.2/10</f>
+        <v>1234.7241191999999</v>
+      </c>
+      <c r="K25" s="20"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" s="30"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="20"/>
+    </row>
+    <row r="27" spans="1:11" ht="69" x14ac:dyDescent="0.3">
+      <c r="A27" s="30">
+        <v>4</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
+      <c r="I27" s="20"/>
+      <c r="J27" s="20"/>
+      <c r="K27" s="20"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="30"/>
+      <c r="B28" s="31" t="str">
+        <f>B10</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C28" s="20">
+        <v>1</v>
+      </c>
+      <c r="D28" s="36">
+        <f>D10</f>
+        <v>39.4</v>
+      </c>
+      <c r="E28" s="20">
+        <v>0.23</v>
+      </c>
+      <c r="F28" s="33">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G28" s="33">
+        <f t="shared" ref="G28:G33" si="0">PRODUCT(C28:F28)</f>
+        <v>0.67964999999999998</v>
+      </c>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="30"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="20">
+        <v>2</v>
+      </c>
+      <c r="D29" s="36">
+        <f>D10</f>
+        <v>39.4</v>
+      </c>
+      <c r="E29" s="20">
+        <v>0.23</v>
+      </c>
+      <c r="F29" s="33">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G29" s="33">
+        <f t="shared" si="0"/>
+        <v>1.3593</v>
+      </c>
+      <c r="H29" s="20"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="20"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="30"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="20">
+        <f>C11</f>
+        <v>16</v>
+      </c>
+      <c r="D30" s="36">
+        <f>D11</f>
+        <v>0.35</v>
+      </c>
+      <c r="E30" s="36">
+        <f>E11</f>
+        <v>0.35</v>
+      </c>
+      <c r="F30" s="36">
+        <v>0.05</v>
+      </c>
+      <c r="G30" s="33">
+        <f t="shared" si="0"/>
+        <v>9.799999999999999E-2</v>
+      </c>
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
+      <c r="K30" s="20"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="30"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="20">
+        <f>C30</f>
+        <v>16</v>
+      </c>
+      <c r="D31" s="36">
+        <v>0.35</v>
+      </c>
+      <c r="E31" s="36">
+        <v>0.35</v>
+      </c>
+      <c r="F31" s="36">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G31" s="33">
+        <f t="shared" si="0"/>
+        <v>0.14699999999999996</v>
+      </c>
+      <c r="H31" s="20"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="30"/>
+      <c r="B32" s="31" t="str">
+        <f>B12</f>
+        <v>-for  stone masonary</v>
+      </c>
+      <c r="C32" s="32">
+        <v>1</v>
+      </c>
+      <c r="D32" s="33">
+        <f>D12</f>
+        <v>45</v>
+      </c>
+      <c r="E32" s="33">
+        <f>F53/2</f>
+        <v>0.5</v>
+      </c>
+      <c r="F32" s="33">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G32" s="33">
+        <f t="shared" si="0"/>
+        <v>1.6875</v>
+      </c>
+      <c r="H32" s="20"/>
+      <c r="I32" s="20"/>
+      <c r="J32" s="20"/>
+      <c r="K32" s="20"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="30"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="32">
+        <v>1</v>
+      </c>
+      <c r="D33" s="33">
+        <f>D32</f>
+        <v>45</v>
+      </c>
+      <c r="E33" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="F33" s="33">
+        <v>0.05</v>
+      </c>
+      <c r="G33" s="33">
+        <f t="shared" si="0"/>
+        <v>1.0125</v>
+      </c>
+      <c r="H33" s="20"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="20"/>
+      <c r="K33" s="20"/>
+    </row>
+    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="8"/>
+      <c r="B34" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="10"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="13">
+        <f>SUM(G28:G33)</f>
+        <v>4.9839499999999992</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I34" s="13">
+        <v>10964.46</v>
+      </c>
+      <c r="J34" s="15">
+        <f>G34*I34</f>
+        <v>54646.320416999988</v>
+      </c>
+      <c r="K34" s="12"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="30"/>
+      <c r="B35" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="20"/>
+      <c r="I35" s="20"/>
+      <c r="J35" s="15">
+        <f>0.13*G34*(119450.3+6325.7)/15</f>
+        <v>5432.797891733333</v>
+      </c>
+      <c r="K35" s="20"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="30"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="20"/>
+      <c r="I36" s="20"/>
+      <c r="J36" s="20"/>
+      <c r="K36" s="20"/>
+    </row>
+    <row r="37" spans="1:11" ht="33" x14ac:dyDescent="0.3">
+      <c r="A37" s="30">
+        <v>5</v>
+      </c>
+      <c r="B37" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="20"/>
+      <c r="I37" s="20"/>
+      <c r="J37" s="20"/>
+      <c r="K37" s="20"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="30"/>
+      <c r="B38" s="31" t="str">
+        <f>B10</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C38" s="32">
+        <v>1</v>
+      </c>
+      <c r="D38" s="33">
+        <f>D10</f>
+        <v>39.4</v>
+      </c>
+      <c r="E38" s="33">
+        <v>0.23</v>
+      </c>
+      <c r="F38" s="33">
+        <f>0.9+0.6-0.075*2</f>
+        <v>1.35</v>
+      </c>
+      <c r="G38" s="33">
+        <f>PRODUCT(C38:F38)</f>
+        <v>12.233700000000001</v>
+      </c>
+      <c r="H38" s="20"/>
+      <c r="I38" s="20"/>
+      <c r="J38" s="20"/>
+      <c r="K38" s="20"/>
+    </row>
+    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="8"/>
+      <c r="B39" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="10"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="13">
+        <f>SUM(G38:G38)</f>
+        <v>12.233700000000001</v>
+      </c>
+      <c r="H39" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I39" s="13">
+        <v>14491.84</v>
+      </c>
+      <c r="J39" s="15">
+        <f>G39*I39</f>
+        <v>177288.82300800001</v>
+      </c>
+      <c r="K39" s="12"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="30"/>
+      <c r="B40" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="20"/>
+      <c r="J40" s="15">
+        <f>0.13*G39*10374.74</f>
+        <v>16499.789375939999</v>
+      </c>
+      <c r="K40" s="20"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="30"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
+      <c r="F41" s="20"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="20"/>
+      <c r="I41" s="20"/>
+      <c r="J41" s="15"/>
+      <c r="K41" s="20"/>
+    </row>
+    <row r="42" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
+      <c r="A42" s="8">
+        <v>6</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C42" s="10"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="40"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="40"/>
+      <c r="K42" s="12"/>
+    </row>
+    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="8"/>
+      <c r="B43" s="41" t="str">
+        <f>B28</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C43" s="10">
+        <v>2</v>
+      </c>
+      <c r="D43" s="11">
+        <f>D38+C11*D11</f>
+        <v>45</v>
+      </c>
+      <c r="E43" s="12"/>
+      <c r="F43" s="12">
+        <v>0.9</v>
+      </c>
+      <c r="G43" s="42">
+        <f t="shared" ref="G43" si="1">PRODUCT(C43:F43)</f>
+        <v>81</v>
+      </c>
+      <c r="H43" s="14"/>
+      <c r="I43" s="13"/>
+      <c r="J43" s="40"/>
+      <c r="K43" s="12"/>
+    </row>
+    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="8"/>
+      <c r="B44" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="C44" s="10"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="12"/>
+      <c r="F44" s="12"/>
+      <c r="G44" s="40">
+        <f>SUM(G41:G43)</f>
+        <v>81</v>
+      </c>
+      <c r="H44" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="I44" s="13">
+        <v>415.5</v>
+      </c>
+      <c r="J44" s="40">
+        <f>G44*I44</f>
+        <v>33655.5</v>
+      </c>
+      <c r="K44" s="12"/>
+    </row>
+    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="8"/>
+      <c r="B45" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="C45" s="10"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="13"/>
+      <c r="J45" s="40">
+        <f>0.13*G44*11650.4/100</f>
+        <v>1226.7871200000002</v>
+      </c>
+      <c r="K45" s="12"/>
+    </row>
+    <row r="46" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A46" s="8"/>
+      <c r="B46" s="39"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="12"/>
+      <c r="G46" s="40"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="40"/>
+      <c r="K46" s="12"/>
+    </row>
+    <row r="47" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
+      <c r="A47" s="8">
+        <v>7</v>
+      </c>
+      <c r="B47" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="C47" s="10"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="40"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="13"/>
+      <c r="J47" s="40"/>
+      <c r="K47" s="12"/>
+    </row>
+    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="8"/>
+      <c r="B48" s="41" t="str">
+        <f>B43</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C48" s="10">
+        <v>2</v>
+      </c>
+      <c r="D48" s="11">
+        <f>D43</f>
+        <v>45</v>
+      </c>
+      <c r="E48" s="12"/>
+      <c r="F48" s="12">
+        <v>0.9</v>
+      </c>
+      <c r="G48" s="42">
+        <f t="shared" ref="G48" si="2">PRODUCT(C48:F48)</f>
+        <v>81</v>
+      </c>
+      <c r="H48" s="14"/>
+      <c r="I48" s="13"/>
+      <c r="J48" s="40"/>
+      <c r="K48" s="12"/>
+    </row>
+    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="8"/>
+      <c r="B49" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="C49" s="10"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="12"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="40">
+        <f>SUM(G46:G48)</f>
+        <v>81</v>
+      </c>
+      <c r="H49" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="I49" s="13">
+        <v>253.8</v>
+      </c>
+      <c r="J49" s="40">
+        <f>G49*I49</f>
+        <v>20557.8</v>
+      </c>
+      <c r="K49" s="12"/>
+    </row>
+    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="8"/>
+      <c r="B50" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" s="10"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="12"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="40"/>
+      <c r="H50" s="14"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="40">
+        <f>0.13*G49*12736/100</f>
+        <v>1341.1008000000002</v>
+      </c>
+      <c r="K50" s="12"/>
+    </row>
+    <row r="51" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+      <c r="A51" s="8"/>
+      <c r="B51" s="39"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="12"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="40"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="40"/>
+      <c r="K51" s="12"/>
+    </row>
+    <row r="52" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
+      <c r="A52" s="30">
+        <v>8</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C52" s="20"/>
+      <c r="D52" s="20"/>
+      <c r="E52" s="20"/>
+      <c r="F52" s="20"/>
+      <c r="G52" s="20"/>
+      <c r="H52" s="20"/>
+      <c r="I52" s="20"/>
+      <c r="J52" s="20"/>
+      <c r="K52" s="20"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" s="30"/>
+      <c r="B53" s="31" t="str">
+        <f>B12</f>
+        <v>-for  stone masonary</v>
+      </c>
+      <c r="C53" s="32">
+        <v>1</v>
+      </c>
+      <c r="D53" s="33">
+        <f>D12</f>
+        <v>45</v>
+      </c>
+      <c r="E53" s="33">
+        <f>((F53/2)+0.45)/2</f>
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="F53" s="33">
+        <v>1</v>
+      </c>
+      <c r="G53" s="33">
+        <f>PRODUCT(C53:F53)</f>
+        <v>21.375</v>
+      </c>
+      <c r="H53" s="20"/>
+      <c r="I53" s="20"/>
+      <c r="J53" s="20"/>
+      <c r="K53" s="20"/>
+    </row>
+    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="8"/>
+      <c r="B54" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54" s="10"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="12"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="13">
+        <f>SUM(G53:G53)</f>
+        <v>21.375</v>
+      </c>
+      <c r="H54" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I54" s="13">
+        <v>9878.43</v>
+      </c>
+      <c r="J54" s="15">
+        <f>G54*I54</f>
+        <v>211151.44125</v>
+      </c>
+      <c r="K54" s="12"/>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" s="30"/>
+      <c r="B55" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="20"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="20"/>
+      <c r="H55" s="20"/>
+      <c r="I55" s="20"/>
+      <c r="J55" s="15">
+        <f>0.13*G54*(27587.1)/5</f>
+        <v>15331.530825</v>
+      </c>
+      <c r="K55" s="20"/>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" s="30"/>
+      <c r="B56" s="20"/>
+      <c r="C56" s="20"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="20"/>
+      <c r="F56" s="20"/>
+      <c r="G56" s="20"/>
+      <c r="H56" s="20"/>
+      <c r="I56" s="20"/>
+      <c r="J56" s="20"/>
+      <c r="K56" s="20"/>
+    </row>
+    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="8">
+        <v>9</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C57" s="10">
+        <v>1</v>
+      </c>
+      <c r="D57" s="11"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="22">
+        <f t="shared" ref="G57" si="3">PRODUCT(C57:F57)</f>
+        <v>1</v>
+      </c>
+      <c r="H57" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I57" s="13">
+        <v>500</v>
+      </c>
+      <c r="J57" s="22">
+        <f>G57*I57</f>
+        <v>500</v>
+      </c>
+      <c r="K57" s="12"/>
+    </row>
+    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="8"/>
+      <c r="B58" s="21"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="12"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="14"/>
+      <c r="I58" s="13"/>
+      <c r="J58" s="15"/>
+      <c r="K58" s="12"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59" s="19"/>
+      <c r="B59" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C59" s="29"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="15"/>
+      <c r="H59" s="15"/>
+      <c r="I59" s="15"/>
+      <c r="J59" s="15">
+        <f>SUM(J13:J57)</f>
+        <v>578400.81454687333</v>
+      </c>
+      <c r="K59" s="17"/>
+    </row>
+    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="23"/>
+      <c r="B61" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="C61" s="43">
+        <f>J59</f>
+        <v>578400.81454687333</v>
+      </c>
+      <c r="D61" s="44"/>
+      <c r="E61" s="38">
+        <v>100</v>
+      </c>
+      <c r="F61" s="23"/>
+      <c r="G61" s="24"/>
+      <c r="H61" s="23"/>
+      <c r="I61" s="25"/>
+      <c r="J61" s="26"/>
+      <c r="K61" s="27"/>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B62" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="C62" s="49">
+        <v>500000</v>
+      </c>
+      <c r="D62" s="50"/>
+      <c r="E62" s="38"/>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B63" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="C63" s="49">
+        <f>C62-C65-C66</f>
+        <v>475000</v>
+      </c>
+      <c r="D63" s="50"/>
+      <c r="E63" s="38">
+        <f>C63/C61*100</f>
+        <v>82.122982550106045</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B64" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="C64" s="55">
+        <f>C61-C63</f>
+        <v>103400.81454687333</v>
+      </c>
+      <c r="D64" s="55"/>
+      <c r="E64" s="38">
+        <f>100-E63</f>
+        <v>17.877017449893955</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B65" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="C65" s="43">
+        <f>C62*0.03</f>
+        <v>15000</v>
+      </c>
+      <c r="D65" s="44"/>
+      <c r="E65" s="38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B66" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="C66" s="43">
+        <f>C62*0.02</f>
+        <v>10000</v>
+      </c>
+      <c r="D66" s="44"/>
+      <c r="E66" s="38">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="C64:D64"/>
+  </mergeCells>
+  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
+  </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="41" max="10" man="1"/>
+  </rowBreaks>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
simple changes for print
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/police chauki.xlsx
+++ b/बजेट माग estimate/police chauki.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB2C47B1-0123-4280-9A9D-D841E6D7DDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040" firstSheet="2" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Estimate (4)" sheetId="10" state="hidden" r:id="rId1"/>
@@ -42,7 +43,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Police sector contribution (2)'!$A$1:$K$66</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Police sector contribution (2)'!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -201,12 +202,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -303,6 +304,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -379,21 +410,21 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -408,7 +439,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -446,7 +477,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -455,7 +486,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -524,6 +555,106 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="19" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -545,7 +676,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -639,7 +770,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -698,9 +829,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -738,9 +869,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -775,7 +906,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -810,7 +941,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -983,22 +1114,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K66"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
@@ -1013,7 +1144,7 @@
       <c r="J1" s="45"/>
       <c r="K1" s="45"/>
     </row>
-    <row r="2" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A2" s="46" t="s">
         <v>1</v>
       </c>
@@ -1028,7 +1159,7 @@
       <c r="J2" s="46"/>
       <c r="K2" s="46"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
         <v>2</v>
       </c>
@@ -1043,7 +1174,7 @@
       <c r="J3" s="47"/>
       <c r="K3" s="47"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
         <v>3</v>
       </c>
@@ -1058,7 +1189,7 @@
       <c r="J4" s="47"/>
       <c r="K4" s="47"/>
     </row>
-    <row r="5" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="48" t="s">
         <v>4</v>
       </c>
@@ -1073,7 +1204,7 @@
       <c r="J5" s="48"/>
       <c r="K5" s="48"/>
     </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="51" t="s">
         <v>42</v>
       </c>
@@ -1090,7 +1221,7 @@
       <c r="J6" s="52"/>
       <c r="K6" s="52"/>
     </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="53" t="s">
         <v>5</v>
       </c>
@@ -1107,7 +1238,7 @@
       <c r="J7" s="54"/>
       <c r="K7" s="54"/>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -1142,7 +1273,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="30">
         <v>1</v>
       </c>
@@ -1159,7 +1290,7 @@
       <c r="J9" s="20"/>
       <c r="K9" s="20"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="30"/>
       <c r="B10" s="31" t="s">
         <v>25</v>
@@ -1186,7 +1317,7 @@
       <c r="J10" s="20"/>
       <c r="K10" s="20"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="30"/>
       <c r="B11" s="31"/>
       <c r="C11" s="32">
@@ -1210,7 +1341,7 @@
       <c r="J11" s="20"/>
       <c r="K11" s="20"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="30"/>
       <c r="B12" s="31" t="s">
         <v>26</v>
@@ -1237,7 +1368,7 @@
       <c r="J12" s="20"/>
       <c r="K12" s="20"/>
     </row>
-    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="9" t="s">
         <v>18</v>
@@ -1262,7 +1393,7 @@
       </c>
       <c r="K13" s="12"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="30"/>
       <c r="B14" s="34" t="s">
         <v>27</v>
@@ -1280,7 +1411,7 @@
       </c>
       <c r="K14" s="20"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="30"/>
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
@@ -1293,7 +1424,7 @@
       <c r="J15" s="20"/>
       <c r="K15" s="20"/>
     </row>
-    <row r="16" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="30">
         <v>2</v>
       </c>
@@ -1310,7 +1441,7 @@
       <c r="J16" s="20"/>
       <c r="K16" s="20"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="30"/>
       <c r="B17" s="31" t="str">
         <f>B12</f>
@@ -1339,7 +1470,7 @@
       <c r="J17" s="20"/>
       <c r="K17" s="20"/>
     </row>
-    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
       <c r="B18" s="9" t="s">
         <v>18</v>
@@ -1364,7 +1495,7 @@
       </c>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="30"/>
       <c r="B19" s="34" t="s">
         <v>27</v>
@@ -1382,7 +1513,7 @@
       </c>
       <c r="K19" s="20"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="30"/>
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
@@ -1395,7 +1526,7 @@
       <c r="J20" s="20"/>
       <c r="K20" s="20"/>
     </row>
-    <row r="21" spans="1:11" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A21" s="30">
         <v>3</v>
       </c>
@@ -1412,7 +1543,7 @@
       <c r="J21" s="20"/>
       <c r="K21" s="20"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="30"/>
       <c r="B22" s="31" t="str">
         <f>B10</f>
@@ -1438,7 +1569,7 @@
       <c r="J22" s="20"/>
       <c r="K22" s="20"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="30"/>
       <c r="B23" s="31"/>
       <c r="C23" s="32">
@@ -1463,7 +1594,7 @@
       <c r="J23" s="20"/>
       <c r="K23" s="20"/>
     </row>
-    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
       <c r="B24" s="9" t="s">
         <v>18</v>
@@ -1488,7 +1619,7 @@
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="30"/>
       <c r="B25" s="34" t="s">
         <v>27</v>
@@ -1506,7 +1637,7 @@
       </c>
       <c r="K25" s="20"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="30"/>
       <c r="B26" s="20"/>
       <c r="C26" s="20"/>
@@ -1519,7 +1650,7 @@
       <c r="J26" s="20"/>
       <c r="K26" s="20"/>
     </row>
-    <row r="27" spans="1:11" ht="69" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A27" s="30">
         <v>4</v>
       </c>
@@ -1536,7 +1667,7 @@
       <c r="J27" s="20"/>
       <c r="K27" s="20"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="30"/>
       <c r="B28" s="31" t="str">
         <f>B10</f>
@@ -1564,7 +1695,7 @@
       <c r="J28" s="20"/>
       <c r="K28" s="20"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="30"/>
       <c r="B29" s="31"/>
       <c r="C29" s="20">
@@ -1589,7 +1720,7 @@
       <c r="J29" s="20"/>
       <c r="K29" s="20"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="30"/>
       <c r="B30" s="31"/>
       <c r="C30" s="20">
@@ -1616,7 +1747,7 @@
       <c r="J30" s="20"/>
       <c r="K30" s="20"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="30"/>
       <c r="B31" s="31"/>
       <c r="C31" s="20">
@@ -1641,7 +1772,7 @@
       <c r="J31" s="20"/>
       <c r="K31" s="20"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="30"/>
       <c r="B32" s="31" t="str">
         <f>B12</f>
@@ -1670,7 +1801,7 @@
       <c r="J32" s="20"/>
       <c r="K32" s="20"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="30"/>
       <c r="B33" s="31"/>
       <c r="C33" s="32">
@@ -1695,7 +1826,7 @@
       <c r="J33" s="20"/>
       <c r="K33" s="20"/>
     </row>
-    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8"/>
       <c r="B34" s="9" t="s">
         <v>18</v>
@@ -1720,7 +1851,7 @@
       </c>
       <c r="K34" s="12"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="30"/>
       <c r="B35" s="34" t="s">
         <v>27</v>
@@ -1738,7 +1869,7 @@
       </c>
       <c r="K35" s="20"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="30"/>
       <c r="B36" s="20"/>
       <c r="C36" s="20"/>
@@ -1751,7 +1882,7 @@
       <c r="J36" s="20"/>
       <c r="K36" s="20"/>
     </row>
-    <row r="37" spans="1:11" ht="33" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="32.25" x14ac:dyDescent="0.25">
       <c r="A37" s="30">
         <v>5</v>
       </c>
@@ -1768,7 +1899,7 @@
       <c r="J37" s="20"/>
       <c r="K37" s="20"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="30"/>
       <c r="B38" s="31" t="str">
         <f>B10</f>
@@ -1797,7 +1928,7 @@
       <c r="J38" s="20"/>
       <c r="K38" s="20"/>
     </row>
-    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8"/>
       <c r="B39" s="9" t="s">
         <v>18</v>
@@ -1822,7 +1953,7 @@
       </c>
       <c r="K39" s="12"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="30"/>
       <c r="B40" s="34" t="s">
         <v>27</v>
@@ -1840,7 +1971,7 @@
       </c>
       <c r="K40" s="20"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="30"/>
       <c r="B41" s="34"/>
       <c r="C41" s="20"/>
@@ -1853,7 +1984,7 @@
       <c r="J41" s="15"/>
       <c r="K41" s="20"/>
     </row>
-    <row r="42" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
       <c r="A42" s="8">
         <v>6</v>
       </c>
@@ -1870,7 +2001,7 @@
       <c r="J42" s="40"/>
       <c r="K42" s="12"/>
     </row>
-    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
       <c r="B43" s="41" t="str">
         <f>B28</f>
@@ -1896,7 +2027,7 @@
       <c r="J43" s="40"/>
       <c r="K43" s="12"/>
     </row>
-    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8"/>
       <c r="B44" s="41" t="s">
         <v>38</v>
@@ -1921,7 +2052,7 @@
       </c>
       <c r="K44" s="12"/>
     </row>
-    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8"/>
       <c r="B45" s="41" t="s">
         <v>40</v>
@@ -1939,7 +2070,7 @@
       </c>
       <c r="K45" s="12"/>
     </row>
-    <row r="46" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="8"/>
       <c r="B46" s="39"/>
       <c r="C46" s="10"/>
@@ -1952,7 +2083,7 @@
       <c r="J46" s="40"/>
       <c r="K46" s="12"/>
     </row>
-    <row r="47" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
       <c r="A47" s="8">
         <v>7</v>
       </c>
@@ -1969,7 +2100,7 @@
       <c r="J47" s="40"/>
       <c r="K47" s="12"/>
     </row>
-    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8"/>
       <c r="B48" s="41" t="str">
         <f>B43</f>
@@ -1995,7 +2126,7 @@
       <c r="J48" s="40"/>
       <c r="K48" s="12"/>
     </row>
-    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8"/>
       <c r="B49" s="41" t="s">
         <v>38</v>
@@ -2020,7 +2151,7 @@
       </c>
       <c r="K49" s="12"/>
     </row>
-    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8"/>
       <c r="B50" s="41" t="s">
         <v>40</v>
@@ -2038,7 +2169,7 @@
       </c>
       <c r="K50" s="12"/>
     </row>
-    <row r="51" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="8"/>
       <c r="B51" s="39"/>
       <c r="C51" s="10"/>
@@ -2051,7 +2182,7 @@
       <c r="J51" s="40"/>
       <c r="K51" s="12"/>
     </row>
-    <row r="52" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A52" s="30">
         <v>8</v>
       </c>
@@ -2068,7 +2199,7 @@
       <c r="J52" s="20"/>
       <c r="K52" s="20"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="30"/>
       <c r="B53" s="31" t="str">
         <f>B12</f>
@@ -2097,7 +2228,7 @@
       <c r="J53" s="20"/>
       <c r="K53" s="20"/>
     </row>
-    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="8"/>
       <c r="B54" s="9" t="s">
         <v>18</v>
@@ -2122,7 +2253,7 @@
       </c>
       <c r="K54" s="12"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="30"/>
       <c r="B55" s="34" t="s">
         <v>27</v>
@@ -2140,7 +2271,7 @@
       </c>
       <c r="K55" s="20"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="30"/>
       <c r="B56" s="20"/>
       <c r="C56" s="20"/>
@@ -2153,7 +2284,7 @@
       <c r="J56" s="20"/>
       <c r="K56" s="20"/>
     </row>
-    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
         <v>9</v>
       </c>
@@ -2182,7 +2313,7 @@
       </c>
       <c r="K57" s="12"/>
     </row>
-    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8"/>
       <c r="B58" s="21"/>
       <c r="C58" s="10"/>
@@ -2195,7 +2326,7 @@
       <c r="J58" s="15"/>
       <c r="K58" s="12"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="19"/>
       <c r="B59" s="28" t="s">
         <v>23</v>
@@ -2213,7 +2344,7 @@
       </c>
       <c r="K59" s="17"/>
     </row>
-    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="23"/>
       <c r="B61" s="37" t="s">
         <v>22</v>
@@ -2233,7 +2364,7 @@
       <c r="J61" s="26"/>
       <c r="K61" s="27"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B62" s="37" t="s">
         <v>33</v>
       </c>
@@ -2243,7 +2374,7 @@
       <c r="D62" s="50"/>
       <c r="E62" s="38"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B63" s="37" t="s">
         <v>34</v>
       </c>
@@ -2257,7 +2388,7 @@
         <v>84.214635175790065</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B64" s="37" t="s">
         <v>32</v>
       </c>
@@ -2271,7 +2402,7 @@
         <v>15.785364824209935</v>
       </c>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="37" t="s">
         <v>35</v>
       </c>
@@ -2284,7 +2415,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" s="37" t="s">
         <v>36</v>
       </c>
@@ -2321,22 +2452,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K66"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
@@ -2351,7 +2482,7 @@
       <c r="J1" s="45"/>
       <c r="K1" s="45"/>
     </row>
-    <row r="2" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A2" s="46" t="s">
         <v>1</v>
       </c>
@@ -2366,7 +2497,7 @@
       <c r="J2" s="46"/>
       <c r="K2" s="46"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
         <v>2</v>
       </c>
@@ -2381,7 +2512,7 @@
       <c r="J3" s="47"/>
       <c r="K3" s="47"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
         <v>3</v>
       </c>
@@ -2396,7 +2527,7 @@
       <c r="J4" s="47"/>
       <c r="K4" s="47"/>
     </row>
-    <row r="5" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="48" t="s">
         <v>4</v>
       </c>
@@ -2411,7 +2542,7 @@
       <c r="J5" s="48"/>
       <c r="K5" s="48"/>
     </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="51" t="s">
         <v>42</v>
       </c>
@@ -2428,7 +2559,7 @@
       <c r="J6" s="52"/>
       <c r="K6" s="52"/>
     </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="53" t="s">
         <v>5</v>
       </c>
@@ -2445,7 +2576,7 @@
       <c r="J7" s="54"/>
       <c r="K7" s="54"/>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -2480,7 +2611,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="124.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="30">
         <v>1</v>
       </c>
@@ -2497,7 +2628,7 @@
       <c r="J9" s="20"/>
       <c r="K9" s="20"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="30"/>
       <c r="B10" s="31" t="s">
         <v>25</v>
@@ -2524,7 +2655,7 @@
       <c r="J10" s="20"/>
       <c r="K10" s="20"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="30"/>
       <c r="B11" s="31"/>
       <c r="C11" s="32">
@@ -2548,7 +2679,7 @@
       <c r="J11" s="20"/>
       <c r="K11" s="20"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="30"/>
       <c r="B12" s="31" t="s">
         <v>26</v>
@@ -2575,7 +2706,7 @@
       <c r="J12" s="20"/>
       <c r="K12" s="20"/>
     </row>
-    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="9" t="s">
         <v>18</v>
@@ -2600,7 +2731,7 @@
       </c>
       <c r="K13" s="12"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="30"/>
       <c r="B14" s="34" t="s">
         <v>27</v>
@@ -2618,7 +2749,7 @@
       </c>
       <c r="K14" s="20"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="30"/>
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
@@ -2631,7 +2762,7 @@
       <c r="J15" s="20"/>
       <c r="K15" s="20"/>
     </row>
-    <row r="16" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A16" s="30">
         <v>2</v>
       </c>
@@ -2648,7 +2779,7 @@
       <c r="J16" s="20"/>
       <c r="K16" s="20"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="30"/>
       <c r="B17" s="31" t="str">
         <f>B12</f>
@@ -2677,7 +2808,7 @@
       <c r="J17" s="20"/>
       <c r="K17" s="20"/>
     </row>
-    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
       <c r="B18" s="9" t="s">
         <v>18</v>
@@ -2702,7 +2833,7 @@
       </c>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="30"/>
       <c r="B19" s="34" t="s">
         <v>27</v>
@@ -2720,7 +2851,7 @@
       </c>
       <c r="K19" s="20"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="30"/>
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
@@ -2733,7 +2864,7 @@
       <c r="J20" s="20"/>
       <c r="K20" s="20"/>
     </row>
-    <row r="21" spans="1:11" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A21" s="30">
         <v>3</v>
       </c>
@@ -2750,7 +2881,7 @@
       <c r="J21" s="20"/>
       <c r="K21" s="20"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="30"/>
       <c r="B22" s="31" t="str">
         <f>B10</f>
@@ -2776,7 +2907,7 @@
       <c r="J22" s="20"/>
       <c r="K22" s="20"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="30"/>
       <c r="B23" s="31"/>
       <c r="C23" s="32">
@@ -2801,7 +2932,7 @@
       <c r="J23" s="20"/>
       <c r="K23" s="20"/>
     </row>
-    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
       <c r="B24" s="9" t="s">
         <v>18</v>
@@ -2826,7 +2957,7 @@
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="30"/>
       <c r="B25" s="34" t="s">
         <v>27</v>
@@ -2844,7 +2975,7 @@
       </c>
       <c r="K25" s="20"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="30"/>
       <c r="B26" s="20"/>
       <c r="C26" s="20"/>
@@ -2857,7 +2988,7 @@
       <c r="J26" s="20"/>
       <c r="K26" s="20"/>
     </row>
-    <row r="27" spans="1:11" ht="69" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A27" s="30">
         <v>4</v>
       </c>
@@ -2874,7 +3005,7 @@
       <c r="J27" s="20"/>
       <c r="K27" s="20"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="30"/>
       <c r="B28" s="31" t="str">
         <f>B10</f>
@@ -2902,7 +3033,7 @@
       <c r="J28" s="20"/>
       <c r="K28" s="20"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="30"/>
       <c r="B29" s="31"/>
       <c r="C29" s="20">
@@ -2927,7 +3058,7 @@
       <c r="J29" s="20"/>
       <c r="K29" s="20"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="30"/>
       <c r="B30" s="31"/>
       <c r="C30" s="20">
@@ -2954,7 +3085,7 @@
       <c r="J30" s="20"/>
       <c r="K30" s="20"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="30"/>
       <c r="B31" s="31"/>
       <c r="C31" s="20">
@@ -2979,7 +3110,7 @@
       <c r="J31" s="20"/>
       <c r="K31" s="20"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="30"/>
       <c r="B32" s="31" t="str">
         <f>B12</f>
@@ -3008,7 +3139,7 @@
       <c r="J32" s="20"/>
       <c r="K32" s="20"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="30"/>
       <c r="B33" s="31"/>
       <c r="C33" s="32">
@@ -3033,7 +3164,7 @@
       <c r="J33" s="20"/>
       <c r="K33" s="20"/>
     </row>
-    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="8"/>
       <c r="B34" s="9" t="s">
         <v>18</v>
@@ -3058,7 +3189,7 @@
       </c>
       <c r="K34" s="12"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="30"/>
       <c r="B35" s="34" t="s">
         <v>27</v>
@@ -3076,7 +3207,7 @@
       </c>
       <c r="K35" s="20"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="30"/>
       <c r="B36" s="20"/>
       <c r="C36" s="20"/>
@@ -3089,7 +3220,7 @@
       <c r="J36" s="20"/>
       <c r="K36" s="20"/>
     </row>
-    <row r="37" spans="1:11" ht="33" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="32.25" x14ac:dyDescent="0.25">
       <c r="A37" s="30">
         <v>5</v>
       </c>
@@ -3106,7 +3237,7 @@
       <c r="J37" s="20"/>
       <c r="K37" s="20"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="30"/>
       <c r="B38" s="31" t="str">
         <f>B10</f>
@@ -3135,7 +3266,7 @@
       <c r="J38" s="20"/>
       <c r="K38" s="20"/>
     </row>
-    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8"/>
       <c r="B39" s="9" t="s">
         <v>18</v>
@@ -3160,7 +3291,7 @@
       </c>
       <c r="K39" s="12"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="30"/>
       <c r="B40" s="34" t="s">
         <v>27</v>
@@ -3178,7 +3309,7 @@
       </c>
       <c r="K40" s="20"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="30"/>
       <c r="B41" s="34"/>
       <c r="C41" s="20"/>
@@ -3191,7 +3322,7 @@
       <c r="J41" s="15"/>
       <c r="K41" s="20"/>
     </row>
-    <row r="42" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
       <c r="A42" s="8">
         <v>6</v>
       </c>
@@ -3208,7 +3339,7 @@
       <c r="J42" s="40"/>
       <c r="K42" s="12"/>
     </row>
-    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
       <c r="B43" s="41" t="str">
         <f>B28</f>
@@ -3234,7 +3365,7 @@
       <c r="J43" s="40"/>
       <c r="K43" s="12"/>
     </row>
-    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8"/>
       <c r="B44" s="41" t="s">
         <v>38</v>
@@ -3259,7 +3390,7 @@
       </c>
       <c r="K44" s="12"/>
     </row>
-    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8"/>
       <c r="B45" s="41" t="s">
         <v>40</v>
@@ -3277,7 +3408,7 @@
       </c>
       <c r="K45" s="12"/>
     </row>
-    <row r="46" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="8"/>
       <c r="B46" s="39"/>
       <c r="C46" s="10"/>
@@ -3290,7 +3421,7 @@
       <c r="J46" s="40"/>
       <c r="K46" s="12"/>
     </row>
-    <row r="47" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" s="16" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
       <c r="A47" s="8">
         <v>7</v>
       </c>
@@ -3307,7 +3438,7 @@
       <c r="J47" s="40"/>
       <c r="K47" s="12"/>
     </row>
-    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8"/>
       <c r="B48" s="41" t="str">
         <f>B43</f>
@@ -3333,7 +3464,7 @@
       <c r="J48" s="40"/>
       <c r="K48" s="12"/>
     </row>
-    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8"/>
       <c r="B49" s="41" t="s">
         <v>38</v>
@@ -3358,7 +3489,7 @@
       </c>
       <c r="K49" s="12"/>
     </row>
-    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8"/>
       <c r="B50" s="41" t="s">
         <v>40</v>
@@ -3376,7 +3507,7 @@
       </c>
       <c r="K50" s="12"/>
     </row>
-    <row r="51" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="8"/>
       <c r="B51" s="39"/>
       <c r="C51" s="10"/>
@@ -3389,7 +3520,7 @@
       <c r="J51" s="40"/>
       <c r="K51" s="12"/>
     </row>
-    <row r="52" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A52" s="30">
         <v>8</v>
       </c>
@@ -3406,7 +3537,7 @@
       <c r="J52" s="20"/>
       <c r="K52" s="20"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="30"/>
       <c r="B53" s="31" t="str">
         <f>B12</f>
@@ -3435,7 +3566,7 @@
       <c r="J53" s="20"/>
       <c r="K53" s="20"/>
     </row>
-    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="8"/>
       <c r="B54" s="9" t="s">
         <v>18</v>
@@ -3460,7 +3591,7 @@
       </c>
       <c r="K54" s="12"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="30"/>
       <c r="B55" s="34" t="s">
         <v>27</v>
@@ -3478,7 +3609,7 @@
       </c>
       <c r="K55" s="20"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="30"/>
       <c r="B56" s="20"/>
       <c r="C56" s="20"/>
@@ -3491,7 +3622,7 @@
       <c r="J56" s="20"/>
       <c r="K56" s="20"/>
     </row>
-    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="8">
         <v>9</v>
       </c>
@@ -3520,7 +3651,7 @@
       </c>
       <c r="K57" s="12"/>
     </row>
-    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="8"/>
       <c r="B58" s="21"/>
       <c r="C58" s="10"/>
@@ -3533,7 +3664,7 @@
       <c r="J58" s="15"/>
       <c r="K58" s="12"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="19"/>
       <c r="B59" s="28" t="s">
         <v>23</v>
@@ -3551,7 +3682,7 @@
       </c>
       <c r="K59" s="17"/>
     </row>
-    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="23"/>
       <c r="B61" s="37" t="s">
         <v>22</v>
@@ -3571,7 +3702,7 @@
       <c r="J61" s="26"/>
       <c r="K61" s="27"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B62" s="37" t="s">
         <v>33</v>
       </c>
@@ -3581,7 +3712,7 @@
       <c r="D62" s="50"/>
       <c r="E62" s="38"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B63" s="37" t="s">
         <v>34</v>
       </c>
@@ -3595,7 +3726,7 @@
         <v>59.555715850778299</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B64" s="37" t="s">
         <v>45</v>
       </c>
@@ -3609,7 +3740,7 @@
         <v>40.444284149221701</v>
       </c>
     </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" s="37" t="s">
         <v>35</v>
       </c>
@@ -3622,7 +3753,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" s="37" t="s">
         <v>36</v>
       </c>
@@ -3632,6 +3763,1361 @@
       </c>
       <c r="D66" s="44"/>
       <c r="E66" s="38">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="C64:D64"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:Q66"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.7109375" style="76" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="76" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" style="76" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" style="76" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="76" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="76" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="76"/>
+    <col min="8" max="8" width="5" style="76" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5703125" style="76" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" style="76" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="76"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="56" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+    </row>
+    <row r="2" spans="1:17" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="57" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="58"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+    </row>
+    <row r="5" spans="1:17" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="59" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="59"/>
+    </row>
+    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="60" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="60"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="62" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" s="62"/>
+      <c r="J6" s="62"/>
+      <c r="K6" s="62"/>
+    </row>
+    <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="63" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="63"/>
+      <c r="C7" s="63"/>
+      <c r="D7" s="63"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="65" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="65"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="65"/>
+    </row>
+    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="66" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="67" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="66" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="68" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="68" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="68" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="66" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="68" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="68" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="69" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="150" x14ac:dyDescent="0.25">
+      <c r="A9" s="70">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="71"/>
+      <c r="D9" s="71"/>
+      <c r="E9" s="71"/>
+      <c r="F9" s="71"/>
+      <c r="G9" s="71"/>
+      <c r="H9" s="71"/>
+      <c r="I9" s="71"/>
+      <c r="J9" s="71"/>
+      <c r="K9" s="71"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="70"/>
+      <c r="B10" s="72" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="71">
+        <v>1</v>
+      </c>
+      <c r="D10" s="73">
+        <f>45-D11*C11</f>
+        <v>39.4</v>
+      </c>
+      <c r="E10" s="73">
+        <v>0.3</v>
+      </c>
+      <c r="F10" s="73">
+        <v>0.75</v>
+      </c>
+      <c r="G10" s="73">
+        <f>PRODUCT(C10:F10)</f>
+        <v>8.8649999999999984</v>
+      </c>
+      <c r="H10" s="71"/>
+      <c r="I10" s="71"/>
+      <c r="J10" s="71"/>
+      <c r="K10" s="71"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="70"/>
+      <c r="B11" s="72"/>
+      <c r="C11" s="71">
+        <f>TRUNC(D17/3,0)+1</f>
+        <v>16</v>
+      </c>
+      <c r="D11" s="73">
+        <v>0.35</v>
+      </c>
+      <c r="E11" s="73">
+        <v>0.35</v>
+      </c>
+      <c r="F11" s="73">
+        <f>F10</f>
+        <v>0.75</v>
+      </c>
+      <c r="G11" s="73">
+        <f>PRODUCT(C11:F11)</f>
+        <v>1.4699999999999998</v>
+      </c>
+      <c r="H11" s="71"/>
+      <c r="I11" s="71"/>
+      <c r="J11" s="71"/>
+      <c r="K11" s="71"/>
+      <c r="O11" s="76">
+        <f>60/2.5</f>
+        <v>24</v>
+      </c>
+      <c r="P11" s="76">
+        <f>60/3</f>
+        <v>20</v>
+      </c>
+      <c r="Q11" s="76">
+        <f>50/3</f>
+        <v>16.666666666666668</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="70"/>
+      <c r="B12" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="71">
+        <v>1</v>
+      </c>
+      <c r="D12" s="73">
+        <v>45</v>
+      </c>
+      <c r="E12" s="73">
+        <f>1.5/2</f>
+        <v>0.75</v>
+      </c>
+      <c r="F12" s="73">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G12" s="73">
+        <f>PRODUCT(C12:F12)</f>
+        <v>33.75</v>
+      </c>
+      <c r="H12" s="71"/>
+      <c r="I12" s="71"/>
+      <c r="J12" s="71"/>
+      <c r="K12" s="71"/>
+    </row>
+    <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8"/>
+      <c r="B13" s="74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="13">
+        <f>SUM(G10:G12)</f>
+        <v>44.084999999999994</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I13" s="13">
+        <v>62.95</v>
+      </c>
+      <c r="J13" s="75">
+        <f>G13*I13</f>
+        <v>2775.1507499999998</v>
+      </c>
+      <c r="K13" s="12"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" s="70"/>
+      <c r="B14" s="72" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="71"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="71"/>
+      <c r="F14" s="71"/>
+      <c r="G14" s="71"/>
+      <c r="H14" s="71"/>
+      <c r="I14" s="71"/>
+      <c r="J14" s="75">
+        <f>0.13*G13*18612/360</f>
+        <v>296.29528499999998</v>
+      </c>
+      <c r="K14" s="71"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" s="70"/>
+      <c r="B15" s="71"/>
+      <c r="C15" s="71"/>
+      <c r="D15" s="71"/>
+      <c r="E15" s="71"/>
+      <c r="F15" s="71"/>
+      <c r="G15" s="71"/>
+      <c r="H15" s="71"/>
+      <c r="I15" s="71"/>
+      <c r="J15" s="71"/>
+      <c r="K15" s="71"/>
+    </row>
+    <row r="16" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+      <c r="A16" s="70">
+        <v>2</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="71"/>
+      <c r="D16" s="71"/>
+      <c r="E16" s="71"/>
+      <c r="F16" s="71"/>
+      <c r="G16" s="71"/>
+      <c r="H16" s="71"/>
+      <c r="I16" s="71"/>
+      <c r="J16" s="71"/>
+      <c r="K16" s="71"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="70"/>
+      <c r="B17" s="72" t="str">
+        <f>B12</f>
+        <v>-for  stone masonary</v>
+      </c>
+      <c r="C17" s="71">
+        <v>1</v>
+      </c>
+      <c r="D17" s="73">
+        <f>D12</f>
+        <v>45</v>
+      </c>
+      <c r="E17" s="73">
+        <f>1.5/2</f>
+        <v>0.75</v>
+      </c>
+      <c r="F17" s="73">
+        <v>0.15</v>
+      </c>
+      <c r="G17" s="73">
+        <f>PRODUCT(C17:F17)</f>
+        <v>5.0625</v>
+      </c>
+      <c r="H17" s="71"/>
+      <c r="I17" s="71"/>
+      <c r="J17" s="71"/>
+      <c r="K17" s="71"/>
+    </row>
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="8"/>
+      <c r="B18" s="74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="13">
+        <f>SUM(G17:G17)</f>
+        <v>5.0625</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I18" s="13">
+        <v>4585.53</v>
+      </c>
+      <c r="J18" s="75">
+        <f>G18*I18</f>
+        <v>23214.245625</v>
+      </c>
+      <c r="K18" s="12"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="70"/>
+      <c r="B19" s="72" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="71"/>
+      <c r="D19" s="71"/>
+      <c r="E19" s="71"/>
+      <c r="F19" s="71"/>
+      <c r="G19" s="71"/>
+      <c r="H19" s="71"/>
+      <c r="I19" s="71"/>
+      <c r="J19" s="75">
+        <f>0.13*G18*15452.64/5</f>
+        <v>2033.9537400000002</v>
+      </c>
+      <c r="K19" s="71"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="70"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="71"/>
+      <c r="F20" s="71"/>
+      <c r="G20" s="71"/>
+      <c r="H20" s="71"/>
+      <c r="I20" s="71"/>
+      <c r="J20" s="71"/>
+      <c r="K20" s="71"/>
+    </row>
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="70">
+        <v>3</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="71"/>
+      <c r="D21" s="71"/>
+      <c r="E21" s="71"/>
+      <c r="F21" s="71"/>
+      <c r="G21" s="71"/>
+      <c r="H21" s="71"/>
+      <c r="I21" s="71"/>
+      <c r="J21" s="71"/>
+      <c r="K21" s="71"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="70"/>
+      <c r="B22" s="72" t="str">
+        <f>B10</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C22" s="71">
+        <v>1</v>
+      </c>
+      <c r="D22" s="73">
+        <f>D10</f>
+        <v>39.4</v>
+      </c>
+      <c r="E22" s="73">
+        <v>0.23</v>
+      </c>
+      <c r="F22" s="73"/>
+      <c r="G22" s="73">
+        <f>PRODUCT(C22:F22)</f>
+        <v>9.0619999999999994</v>
+      </c>
+      <c r="H22" s="71"/>
+      <c r="I22" s="71"/>
+      <c r="J22" s="71"/>
+      <c r="K22" s="71"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="70"/>
+      <c r="B23" s="72"/>
+      <c r="C23" s="71">
+        <f>C11</f>
+        <v>16</v>
+      </c>
+      <c r="D23" s="73">
+        <f>D11</f>
+        <v>0.35</v>
+      </c>
+      <c r="E23" s="73">
+        <f>E11</f>
+        <v>0.35</v>
+      </c>
+      <c r="F23" s="73"/>
+      <c r="G23" s="73">
+        <f>PRODUCT(C23:F23)</f>
+        <v>1.9599999999999997</v>
+      </c>
+      <c r="H23" s="71"/>
+      <c r="I23" s="71"/>
+      <c r="J23" s="71"/>
+      <c r="K23" s="71"/>
+    </row>
+    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="8"/>
+      <c r="B24" s="74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="13">
+        <f>SUM(G22:G23)</f>
+        <v>11.021999999999998</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I24" s="13">
+        <v>1017.47</v>
+      </c>
+      <c r="J24" s="75">
+        <f>G24*I24</f>
+        <v>11214.554339999999</v>
+      </c>
+      <c r="K24" s="12"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="70"/>
+      <c r="B25" s="72" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="71"/>
+      <c r="D25" s="71"/>
+      <c r="E25" s="71"/>
+      <c r="F25" s="71"/>
+      <c r="G25" s="71"/>
+      <c r="H25" s="71"/>
+      <c r="I25" s="71"/>
+      <c r="J25" s="75">
+        <f>0.13*G24*8617.2/10</f>
+        <v>1234.7241191999999</v>
+      </c>
+      <c r="K25" s="71"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="70"/>
+      <c r="B26" s="71"/>
+      <c r="C26" s="71"/>
+      <c r="D26" s="71"/>
+      <c r="E26" s="71"/>
+      <c r="F26" s="71"/>
+      <c r="G26" s="71"/>
+      <c r="H26" s="71"/>
+      <c r="I26" s="71"/>
+      <c r="J26" s="71"/>
+      <c r="K26" s="71"/>
+    </row>
+    <row r="27" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+      <c r="A27" s="70">
+        <v>4</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="71"/>
+      <c r="D27" s="71"/>
+      <c r="E27" s="71"/>
+      <c r="F27" s="71"/>
+      <c r="G27" s="71"/>
+      <c r="H27" s="71"/>
+      <c r="I27" s="71"/>
+      <c r="J27" s="71"/>
+      <c r="K27" s="71"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="70"/>
+      <c r="B28" s="72" t="str">
+        <f>B10</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C28" s="71">
+        <v>1</v>
+      </c>
+      <c r="D28" s="73">
+        <f>D10</f>
+        <v>39.4</v>
+      </c>
+      <c r="E28" s="71">
+        <v>0.23</v>
+      </c>
+      <c r="F28" s="73">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G28" s="73">
+        <f t="shared" ref="G28:G33" si="0">PRODUCT(C28:F28)</f>
+        <v>0.67964999999999998</v>
+      </c>
+      <c r="H28" s="71"/>
+      <c r="I28" s="71"/>
+      <c r="J28" s="71"/>
+      <c r="K28" s="71"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="70"/>
+      <c r="B29" s="72"/>
+      <c r="C29" s="71">
+        <v>2</v>
+      </c>
+      <c r="D29" s="73">
+        <f>D10</f>
+        <v>39.4</v>
+      </c>
+      <c r="E29" s="71">
+        <v>0.23</v>
+      </c>
+      <c r="F29" s="73">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G29" s="73">
+        <f t="shared" si="0"/>
+        <v>1.3593</v>
+      </c>
+      <c r="H29" s="71"/>
+      <c r="I29" s="71"/>
+      <c r="J29" s="71"/>
+      <c r="K29" s="71"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="70"/>
+      <c r="B30" s="72"/>
+      <c r="C30" s="71">
+        <f>C11</f>
+        <v>16</v>
+      </c>
+      <c r="D30" s="73">
+        <f>D11</f>
+        <v>0.35</v>
+      </c>
+      <c r="E30" s="73">
+        <f>E11</f>
+        <v>0.35</v>
+      </c>
+      <c r="F30" s="73">
+        <v>0.05</v>
+      </c>
+      <c r="G30" s="73">
+        <f t="shared" si="0"/>
+        <v>9.799999999999999E-2</v>
+      </c>
+      <c r="H30" s="71"/>
+      <c r="I30" s="71"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="71"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="70"/>
+      <c r="B31" s="72"/>
+      <c r="C31" s="71">
+        <f>C30</f>
+        <v>16</v>
+      </c>
+      <c r="D31" s="73">
+        <v>0.35</v>
+      </c>
+      <c r="E31" s="73">
+        <v>0.35</v>
+      </c>
+      <c r="F31" s="73">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G31" s="73">
+        <f t="shared" si="0"/>
+        <v>0.14699999999999996</v>
+      </c>
+      <c r="H31" s="71"/>
+      <c r="I31" s="71"/>
+      <c r="J31" s="71"/>
+      <c r="K31" s="71"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="70"/>
+      <c r="B32" s="72" t="str">
+        <f>B12</f>
+        <v>-for  stone masonary</v>
+      </c>
+      <c r="C32" s="71">
+        <v>1</v>
+      </c>
+      <c r="D32" s="73">
+        <f>D12</f>
+        <v>45</v>
+      </c>
+      <c r="E32" s="73">
+        <f>F53/2</f>
+        <v>0.5</v>
+      </c>
+      <c r="F32" s="73">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G32" s="73">
+        <f t="shared" si="0"/>
+        <v>1.6875</v>
+      </c>
+      <c r="H32" s="71"/>
+      <c r="I32" s="71"/>
+      <c r="J32" s="71"/>
+      <c r="K32" s="71"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="70"/>
+      <c r="B33" s="72"/>
+      <c r="C33" s="71">
+        <v>1</v>
+      </c>
+      <c r="D33" s="73">
+        <f>D32</f>
+        <v>45</v>
+      </c>
+      <c r="E33" s="73">
+        <v>0.45</v>
+      </c>
+      <c r="F33" s="73">
+        <v>0.05</v>
+      </c>
+      <c r="G33" s="73">
+        <f t="shared" si="0"/>
+        <v>1.0125</v>
+      </c>
+      <c r="H33" s="71"/>
+      <c r="I33" s="71"/>
+      <c r="J33" s="71"/>
+      <c r="K33" s="71"/>
+    </row>
+    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="8"/>
+      <c r="B34" s="74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="10"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="13">
+        <f>SUM(G28:G33)</f>
+        <v>4.9839499999999992</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I34" s="13">
+        <v>10964.46</v>
+      </c>
+      <c r="J34" s="75">
+        <f>G34*I34</f>
+        <v>54646.320416999988</v>
+      </c>
+      <c r="K34" s="12"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="70"/>
+      <c r="B35" s="72" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="71"/>
+      <c r="D35" s="71"/>
+      <c r="E35" s="71"/>
+      <c r="F35" s="71"/>
+      <c r="G35" s="71"/>
+      <c r="H35" s="71"/>
+      <c r="I35" s="71"/>
+      <c r="J35" s="75">
+        <f>0.13*G34*(119450.3+6325.7)/15</f>
+        <v>5432.797891733333</v>
+      </c>
+      <c r="K35" s="71"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="70"/>
+      <c r="B36" s="71"/>
+      <c r="C36" s="71"/>
+      <c r="D36" s="71"/>
+      <c r="E36" s="71"/>
+      <c r="F36" s="71"/>
+      <c r="G36" s="71"/>
+      <c r="H36" s="71"/>
+      <c r="I36" s="71"/>
+      <c r="J36" s="71"/>
+      <c r="K36" s="71"/>
+    </row>
+    <row r="37" spans="1:11" ht="32.25" x14ac:dyDescent="0.25">
+      <c r="A37" s="70">
+        <v>5</v>
+      </c>
+      <c r="B37" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="71"/>
+      <c r="D37" s="71"/>
+      <c r="E37" s="71"/>
+      <c r="F37" s="71"/>
+      <c r="G37" s="71"/>
+      <c r="H37" s="71"/>
+      <c r="I37" s="71"/>
+      <c r="J37" s="71"/>
+      <c r="K37" s="71"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="70"/>
+      <c r="B38" s="72" t="str">
+        <f>B10</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C38" s="71">
+        <v>1</v>
+      </c>
+      <c r="D38" s="73">
+        <f>D10</f>
+        <v>39.4</v>
+      </c>
+      <c r="E38" s="73">
+        <v>0.23</v>
+      </c>
+      <c r="F38" s="73">
+        <f>0.9+0.6-0.075*2</f>
+        <v>1.35</v>
+      </c>
+      <c r="G38" s="73">
+        <f>PRODUCT(C38:F38)</f>
+        <v>12.233700000000001</v>
+      </c>
+      <c r="H38" s="71"/>
+      <c r="I38" s="71"/>
+      <c r="J38" s="71"/>
+      <c r="K38" s="71"/>
+    </row>
+    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="8"/>
+      <c r="B39" s="74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="10"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="13">
+        <f>SUM(G38:G38)</f>
+        <v>12.233700000000001</v>
+      </c>
+      <c r="H39" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I39" s="13">
+        <v>14491.84</v>
+      </c>
+      <c r="J39" s="75">
+        <f>G39*I39</f>
+        <v>177288.82300800001</v>
+      </c>
+      <c r="K39" s="12"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="70"/>
+      <c r="B40" s="72" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" s="71"/>
+      <c r="D40" s="71"/>
+      <c r="E40" s="71"/>
+      <c r="F40" s="71"/>
+      <c r="G40" s="71"/>
+      <c r="H40" s="71"/>
+      <c r="I40" s="71"/>
+      <c r="J40" s="75">
+        <f>0.13*G39*10374.74</f>
+        <v>16499.789375939999</v>
+      </c>
+      <c r="K40" s="71"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="70"/>
+      <c r="B41" s="72"/>
+      <c r="C41" s="71"/>
+      <c r="D41" s="71"/>
+      <c r="E41" s="71"/>
+      <c r="F41" s="71"/>
+      <c r="G41" s="71"/>
+      <c r="H41" s="71"/>
+      <c r="I41" s="71"/>
+      <c r="J41" s="75"/>
+      <c r="K41" s="71"/>
+    </row>
+    <row r="42" spans="1:11" s="78" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+      <c r="A42" s="8">
+        <v>6</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C42" s="10"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="77"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="77"/>
+      <c r="K42" s="12"/>
+    </row>
+    <row r="43" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="8"/>
+      <c r="B43" s="79" t="str">
+        <f>B28</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C43" s="10">
+        <v>2</v>
+      </c>
+      <c r="D43" s="11">
+        <f>D38+C11*D11</f>
+        <v>45</v>
+      </c>
+      <c r="E43" s="12"/>
+      <c r="F43" s="12">
+        <v>0.9</v>
+      </c>
+      <c r="G43" s="42">
+        <f t="shared" ref="G43" si="1">PRODUCT(C43:F43)</f>
+        <v>81</v>
+      </c>
+      <c r="H43" s="14"/>
+      <c r="I43" s="13"/>
+      <c r="J43" s="77"/>
+      <c r="K43" s="12"/>
+    </row>
+    <row r="44" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="8"/>
+      <c r="B44" s="79" t="s">
+        <v>38</v>
+      </c>
+      <c r="C44" s="10"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="12"/>
+      <c r="F44" s="12"/>
+      <c r="G44" s="77">
+        <f>SUM(G41:G43)</f>
+        <v>81</v>
+      </c>
+      <c r="H44" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="I44" s="13">
+        <v>415.5</v>
+      </c>
+      <c r="J44" s="77">
+        <f>G44*I44</f>
+        <v>33655.5</v>
+      </c>
+      <c r="K44" s="12"/>
+    </row>
+    <row r="45" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="8"/>
+      <c r="B45" s="79" t="s">
+        <v>40</v>
+      </c>
+      <c r="C45" s="10"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="77"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="13"/>
+      <c r="J45" s="77">
+        <f>0.13*G44*11650.4/100</f>
+        <v>1226.7871200000002</v>
+      </c>
+      <c r="K45" s="12"/>
+    </row>
+    <row r="46" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="8"/>
+      <c r="B46" s="39"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="12"/>
+      <c r="G46" s="77"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="77"/>
+      <c r="K46" s="12"/>
+    </row>
+    <row r="47" spans="1:11" s="78" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+      <c r="A47" s="8">
+        <v>7</v>
+      </c>
+      <c r="B47" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="C47" s="10"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="77"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="13"/>
+      <c r="J47" s="77"/>
+      <c r="K47" s="12"/>
+    </row>
+    <row r="48" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="8"/>
+      <c r="B48" s="79" t="str">
+        <f>B43</f>
+        <v>-for brick wall</v>
+      </c>
+      <c r="C48" s="10">
+        <v>2</v>
+      </c>
+      <c r="D48" s="11">
+        <f>D43</f>
+        <v>45</v>
+      </c>
+      <c r="E48" s="12"/>
+      <c r="F48" s="12">
+        <v>0.9</v>
+      </c>
+      <c r="G48" s="42">
+        <f t="shared" ref="G48" si="2">PRODUCT(C48:F48)</f>
+        <v>81</v>
+      </c>
+      <c r="H48" s="14"/>
+      <c r="I48" s="13"/>
+      <c r="J48" s="77"/>
+      <c r="K48" s="12"/>
+    </row>
+    <row r="49" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="8"/>
+      <c r="B49" s="79" t="s">
+        <v>38</v>
+      </c>
+      <c r="C49" s="10"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="12"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="77">
+        <f>SUM(G46:G48)</f>
+        <v>81</v>
+      </c>
+      <c r="H49" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="I49" s="13">
+        <v>253.8</v>
+      </c>
+      <c r="J49" s="77">
+        <f>G49*I49</f>
+        <v>20557.8</v>
+      </c>
+      <c r="K49" s="12"/>
+    </row>
+    <row r="50" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="8"/>
+      <c r="B50" s="79" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" s="10"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="12"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="77"/>
+      <c r="H50" s="14"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="77">
+        <f>0.13*G49*12736/100</f>
+        <v>1341.1008000000002</v>
+      </c>
+      <c r="K50" s="12"/>
+    </row>
+    <row r="51" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="8"/>
+      <c r="B51" s="39"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="12"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="77"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="77"/>
+      <c r="K51" s="12"/>
+    </row>
+    <row r="52" spans="1:11" ht="90" x14ac:dyDescent="0.25">
+      <c r="A52" s="70">
+        <v>8</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C52" s="71"/>
+      <c r="D52" s="71"/>
+      <c r="E52" s="71"/>
+      <c r="F52" s="71"/>
+      <c r="G52" s="71"/>
+      <c r="H52" s="71"/>
+      <c r="I52" s="71"/>
+      <c r="J52" s="71"/>
+      <c r="K52" s="71"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="70"/>
+      <c r="B53" s="72" t="str">
+        <f>B12</f>
+        <v>-for  stone masonary</v>
+      </c>
+      <c r="C53" s="71">
+        <v>1</v>
+      </c>
+      <c r="D53" s="73">
+        <f>D12</f>
+        <v>45</v>
+      </c>
+      <c r="E53" s="73">
+        <f>((F53/2)+0.45)/2</f>
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="F53" s="73">
+        <v>1</v>
+      </c>
+      <c r="G53" s="73">
+        <f>PRODUCT(C53:F53)</f>
+        <v>21.375</v>
+      </c>
+      <c r="H53" s="71"/>
+      <c r="I53" s="71"/>
+      <c r="J53" s="71"/>
+      <c r="K53" s="71"/>
+    </row>
+    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="8"/>
+      <c r="B54" s="74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54" s="10"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="12"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="13">
+        <f>SUM(G53:G53)</f>
+        <v>21.375</v>
+      </c>
+      <c r="H54" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="I54" s="13">
+        <v>9878.43</v>
+      </c>
+      <c r="J54" s="75">
+        <f>G54*I54</f>
+        <v>211151.44125</v>
+      </c>
+      <c r="K54" s="12"/>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="70"/>
+      <c r="B55" s="72" t="s">
+        <v>27</v>
+      </c>
+      <c r="C55" s="71"/>
+      <c r="D55" s="71"/>
+      <c r="E55" s="71"/>
+      <c r="F55" s="71"/>
+      <c r="G55" s="71"/>
+      <c r="H55" s="71"/>
+      <c r="I55" s="71"/>
+      <c r="J55" s="75">
+        <f>0.13*G54*(27587.1)/5</f>
+        <v>15331.530825</v>
+      </c>
+      <c r="K55" s="71"/>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="70"/>
+      <c r="B56" s="71"/>
+      <c r="C56" s="71"/>
+      <c r="D56" s="71"/>
+      <c r="E56" s="71"/>
+      <c r="F56" s="71"/>
+      <c r="G56" s="71"/>
+      <c r="H56" s="71"/>
+      <c r="I56" s="71"/>
+      <c r="J56" s="71"/>
+      <c r="K56" s="71"/>
+    </row>
+    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="8">
+        <v>9</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C57" s="10">
+        <v>1</v>
+      </c>
+      <c r="D57" s="11"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="14">
+        <f t="shared" ref="G57" si="3">PRODUCT(C57:F57)</f>
+        <v>1</v>
+      </c>
+      <c r="H57" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I57" s="13">
+        <v>500</v>
+      </c>
+      <c r="J57" s="14">
+        <f>G57*I57</f>
+        <v>500</v>
+      </c>
+      <c r="K57" s="12"/>
+    </row>
+    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="8"/>
+      <c r="B58" s="21"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="12"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="14"/>
+      <c r="I58" s="13"/>
+      <c r="J58" s="75"/>
+      <c r="K58" s="12"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="80"/>
+      <c r="B59" s="81" t="s">
+        <v>23</v>
+      </c>
+      <c r="C59" s="82"/>
+      <c r="D59" s="83"/>
+      <c r="E59" s="83"/>
+      <c r="F59" s="83"/>
+      <c r="G59" s="75"/>
+      <c r="H59" s="75"/>
+      <c r="I59" s="75"/>
+      <c r="J59" s="75">
+        <f>SUM(J13:J57)</f>
+        <v>578400.81454687333</v>
+      </c>
+      <c r="K59" s="84"/>
+    </row>
+    <row r="61" spans="1:11" s="78" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="85"/>
+      <c r="B61" s="86" t="s">
+        <v>22</v>
+      </c>
+      <c r="C61" s="87">
+        <f>J59</f>
+        <v>578400.81454687333</v>
+      </c>
+      <c r="D61" s="88"/>
+      <c r="E61" s="42">
+        <v>100</v>
+      </c>
+      <c r="F61" s="85"/>
+      <c r="G61" s="89"/>
+      <c r="H61" s="85"/>
+      <c r="I61" s="90"/>
+      <c r="J61" s="91"/>
+      <c r="K61" s="92"/>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B62" s="86" t="s">
+        <v>33</v>
+      </c>
+      <c r="C62" s="93">
+        <v>500000</v>
+      </c>
+      <c r="D62" s="94"/>
+      <c r="E62" s="42"/>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B63" s="86" t="s">
+        <v>34</v>
+      </c>
+      <c r="C63" s="93">
+        <f>C62-C65-C66</f>
+        <v>475000</v>
+      </c>
+      <c r="D63" s="94"/>
+      <c r="E63" s="42">
+        <f>C63/C61*100</f>
+        <v>82.122982550106045</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B64" s="86" t="s">
+        <v>45</v>
+      </c>
+      <c r="C64" s="95">
+        <f>C61-C63</f>
+        <v>103400.81454687333</v>
+      </c>
+      <c r="D64" s="95"/>
+      <c r="E64" s="42">
+        <f>100-E63</f>
+        <v>17.877017449893955</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B65" s="86" t="s">
+        <v>35</v>
+      </c>
+      <c r="C65" s="87">
+        <f>C62*0.03</f>
+        <v>15000</v>
+      </c>
+      <c r="D65" s="88"/>
+      <c r="E65" s="42">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B66" s="86" t="s">
+        <v>36</v>
+      </c>
+      <c r="C66" s="87">
+        <f>C62*0.02</f>
+        <v>10000</v>
+      </c>
+      <c r="D66" s="88"/>
+      <c r="E66" s="42">
         <v>2</v>
       </c>
     </row>
@@ -3653,1359 +5139,6 @@
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q66"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="4.6640625" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" customWidth="1"/>
-    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.88671875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-    </row>
-    <row r="2" spans="1:17" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="46" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" s="47" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47"/>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47"/>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" s="47" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="47"/>
-      <c r="F4" s="47"/>
-      <c r="G4" s="47"/>
-      <c r="H4" s="47"/>
-      <c r="I4" s="47"/>
-      <c r="J4" s="47"/>
-      <c r="K4" s="47"/>
-    </row>
-    <row r="5" spans="1:17" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="48" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48"/>
-    </row>
-    <row r="6" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="51" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="52" t="s">
-        <v>43</v>
-      </c>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="52"/>
-    </row>
-    <row r="7" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="53" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="54" t="s">
-        <v>24</v>
-      </c>
-      <c r="I7" s="54"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="54"/>
-    </row>
-    <row r="8" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" ht="124.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="30">
-        <v>1</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
-      <c r="J9" s="20"/>
-      <c r="K9" s="20"/>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A10" s="30"/>
-      <c r="B10" s="31" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="32">
-        <v>1</v>
-      </c>
-      <c r="D10" s="33">
-        <f>45-D11*C11</f>
-        <v>39.4</v>
-      </c>
-      <c r="E10" s="33">
-        <v>0.3</v>
-      </c>
-      <c r="F10" s="33">
-        <v>0.75</v>
-      </c>
-      <c r="G10" s="33">
-        <f>PRODUCT(C10:F10)</f>
-        <v>8.8649999999999984</v>
-      </c>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A11" s="30"/>
-      <c r="B11" s="31"/>
-      <c r="C11" s="32">
-        <f>TRUNC(D17/3,0)+1</f>
-        <v>16</v>
-      </c>
-      <c r="D11" s="33">
-        <v>0.35</v>
-      </c>
-      <c r="E11" s="33">
-        <v>0.35</v>
-      </c>
-      <c r="F11" s="33">
-        <f>F10</f>
-        <v>0.75</v>
-      </c>
-      <c r="G11" s="33">
-        <f>PRODUCT(C11:F11)</f>
-        <v>1.4699999999999998</v>
-      </c>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20"/>
-      <c r="O11">
-        <f>60/2.5</f>
-        <v>24</v>
-      </c>
-      <c r="P11">
-        <f>60/3</f>
-        <v>20</v>
-      </c>
-      <c r="Q11">
-        <f>50/3</f>
-        <v>16.666666666666668</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A12" s="30"/>
-      <c r="B12" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="32">
-        <v>1</v>
-      </c>
-      <c r="D12" s="33">
-        <v>45</v>
-      </c>
-      <c r="E12" s="33">
-        <f>1.5/2</f>
-        <v>0.75</v>
-      </c>
-      <c r="F12" s="33">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="G12" s="33">
-        <f>PRODUCT(C12:F12)</f>
-        <v>33.75</v>
-      </c>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
-    </row>
-    <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8"/>
-      <c r="B13" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="13">
-        <f>SUM(G10:G12)</f>
-        <v>44.084999999999994</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I13" s="13">
-        <v>62.95</v>
-      </c>
-      <c r="J13" s="15">
-        <f>G13*I13</f>
-        <v>2775.1507499999998</v>
-      </c>
-      <c r="K13" s="12"/>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A14" s="30"/>
-      <c r="B14" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="15">
-        <f>0.13*G13*18612/360</f>
-        <v>296.29528499999998</v>
-      </c>
-      <c r="K14" s="20"/>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A15" s="30"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
-      <c r="K15" s="20"/>
-    </row>
-    <row r="16" spans="1:17" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="30">
-        <v>2</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="30"/>
-      <c r="B17" s="31" t="str">
-        <f>B12</f>
-        <v>-for  stone masonary</v>
-      </c>
-      <c r="C17" s="32">
-        <v>1</v>
-      </c>
-      <c r="D17" s="33">
-        <f>D12</f>
-        <v>45</v>
-      </c>
-      <c r="E17" s="33">
-        <f>1.5/2</f>
-        <v>0.75</v>
-      </c>
-      <c r="F17" s="33">
-        <v>0.15</v>
-      </c>
-      <c r="G17" s="33">
-        <f>PRODUCT(C17:F17)</f>
-        <v>5.0625</v>
-      </c>
-      <c r="H17" s="20"/>
-      <c r="I17" s="20"/>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20"/>
-    </row>
-    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8"/>
-      <c r="B18" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="13">
-        <f>SUM(G17:G17)</f>
-        <v>5.0625</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I18" s="13">
-        <v>4585.53</v>
-      </c>
-      <c r="J18" s="15">
-        <f>G18*I18</f>
-        <v>23214.245625</v>
-      </c>
-      <c r="K18" s="12"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="30"/>
-      <c r="B19" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="15">
-        <f>0.13*G18*15452.64/5</f>
-        <v>2033.9537400000002</v>
-      </c>
-      <c r="K19" s="20"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="30"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20"/>
-    </row>
-    <row r="21" spans="1:11" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="30">
-        <v>3</v>
-      </c>
-      <c r="B21" s="35" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="30"/>
-      <c r="B22" s="31" t="str">
-        <f>B10</f>
-        <v>-for brick wall</v>
-      </c>
-      <c r="C22" s="32">
-        <v>1</v>
-      </c>
-      <c r="D22" s="33">
-        <f>D10</f>
-        <v>39.4</v>
-      </c>
-      <c r="E22" s="33">
-        <v>0.23</v>
-      </c>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33">
-        <f>PRODUCT(C22:F22)</f>
-        <v>9.0619999999999994</v>
-      </c>
-      <c r="H22" s="20"/>
-      <c r="I22" s="20"/>
-      <c r="J22" s="20"/>
-      <c r="K22" s="20"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" s="30"/>
-      <c r="B23" s="31"/>
-      <c r="C23" s="32">
-        <f>C11</f>
-        <v>16</v>
-      </c>
-      <c r="D23" s="33">
-        <f>D11</f>
-        <v>0.35</v>
-      </c>
-      <c r="E23" s="33">
-        <f>E11</f>
-        <v>0.35</v>
-      </c>
-      <c r="F23" s="33"/>
-      <c r="G23" s="33">
-        <f>PRODUCT(C23:F23)</f>
-        <v>1.9599999999999997</v>
-      </c>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
-    </row>
-    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="8"/>
-      <c r="B24" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="13">
-        <f>SUM(G22:G23)</f>
-        <v>11.021999999999998</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I24" s="13">
-        <v>1017.47</v>
-      </c>
-      <c r="J24" s="15">
-        <f>G24*I24</f>
-        <v>11214.554339999999</v>
-      </c>
-      <c r="K24" s="12"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" s="30"/>
-      <c r="B25" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="20"/>
-      <c r="J25" s="15">
-        <f>0.13*G24*8617.2/10</f>
-        <v>1234.7241191999999</v>
-      </c>
-      <c r="K25" s="20"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" s="30"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="20"/>
-      <c r="J26" s="20"/>
-      <c r="K26" s="20"/>
-    </row>
-    <row r="27" spans="1:11" ht="69" x14ac:dyDescent="0.3">
-      <c r="A27" s="30">
-        <v>4</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="20"/>
-      <c r="J27" s="20"/>
-      <c r="K27" s="20"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A28" s="30"/>
-      <c r="B28" s="31" t="str">
-        <f>B10</f>
-        <v>-for brick wall</v>
-      </c>
-      <c r="C28" s="20">
-        <v>1</v>
-      </c>
-      <c r="D28" s="36">
-        <f>D10</f>
-        <v>39.4</v>
-      </c>
-      <c r="E28" s="20">
-        <v>0.23</v>
-      </c>
-      <c r="F28" s="33">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="G28" s="33">
-        <f t="shared" ref="G28:G33" si="0">PRODUCT(C28:F28)</f>
-        <v>0.67964999999999998</v>
-      </c>
-      <c r="H28" s="20"/>
-      <c r="I28" s="20"/>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" s="30"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="20">
-        <v>2</v>
-      </c>
-      <c r="D29" s="36">
-        <f>D10</f>
-        <v>39.4</v>
-      </c>
-      <c r="E29" s="20">
-        <v>0.23</v>
-      </c>
-      <c r="F29" s="33">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="G29" s="33">
-        <f t="shared" si="0"/>
-        <v>1.3593</v>
-      </c>
-      <c r="H29" s="20"/>
-      <c r="I29" s="20"/>
-      <c r="J29" s="20"/>
-      <c r="K29" s="20"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A30" s="30"/>
-      <c r="B30" s="31"/>
-      <c r="C30" s="20">
-        <f>C11</f>
-        <v>16</v>
-      </c>
-      <c r="D30" s="36">
-        <f>D11</f>
-        <v>0.35</v>
-      </c>
-      <c r="E30" s="36">
-        <f>E11</f>
-        <v>0.35</v>
-      </c>
-      <c r="F30" s="36">
-        <v>0.05</v>
-      </c>
-      <c r="G30" s="33">
-        <f t="shared" si="0"/>
-        <v>9.799999999999999E-2</v>
-      </c>
-      <c r="H30" s="20"/>
-      <c r="I30" s="20"/>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="30"/>
-      <c r="B31" s="31"/>
-      <c r="C31" s="20">
-        <f>C30</f>
-        <v>16</v>
-      </c>
-      <c r="D31" s="36">
-        <v>0.35</v>
-      </c>
-      <c r="E31" s="36">
-        <v>0.35</v>
-      </c>
-      <c r="F31" s="36">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="G31" s="33">
-        <f t="shared" si="0"/>
-        <v>0.14699999999999996</v>
-      </c>
-      <c r="H31" s="20"/>
-      <c r="I31" s="20"/>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="30"/>
-      <c r="B32" s="31" t="str">
-        <f>B12</f>
-        <v>-for  stone masonary</v>
-      </c>
-      <c r="C32" s="32">
-        <v>1</v>
-      </c>
-      <c r="D32" s="33">
-        <f>D12</f>
-        <v>45</v>
-      </c>
-      <c r="E32" s="33">
-        <f>F53/2</f>
-        <v>0.5</v>
-      </c>
-      <c r="F32" s="33">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="G32" s="33">
-        <f t="shared" si="0"/>
-        <v>1.6875</v>
-      </c>
-      <c r="H32" s="20"/>
-      <c r="I32" s="20"/>
-      <c r="J32" s="20"/>
-      <c r="K32" s="20"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="30"/>
-      <c r="B33" s="31"/>
-      <c r="C33" s="32">
-        <v>1</v>
-      </c>
-      <c r="D33" s="33">
-        <f>D32</f>
-        <v>45</v>
-      </c>
-      <c r="E33" s="33">
-        <v>0.45</v>
-      </c>
-      <c r="F33" s="33">
-        <v>0.05</v>
-      </c>
-      <c r="G33" s="33">
-        <f t="shared" si="0"/>
-        <v>1.0125</v>
-      </c>
-      <c r="H33" s="20"/>
-      <c r="I33" s="20"/>
-      <c r="J33" s="20"/>
-      <c r="K33" s="20"/>
-    </row>
-    <row r="34" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8"/>
-      <c r="B34" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C34" s="10"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="13">
-        <f>SUM(G28:G33)</f>
-        <v>4.9839499999999992</v>
-      </c>
-      <c r="H34" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I34" s="13">
-        <v>10964.46</v>
-      </c>
-      <c r="J34" s="15">
-        <f>G34*I34</f>
-        <v>54646.320416999988</v>
-      </c>
-      <c r="K34" s="12"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A35" s="30"/>
-      <c r="B35" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="20"/>
-      <c r="J35" s="15">
-        <f>0.13*G34*(119450.3+6325.7)/15</f>
-        <v>5432.797891733333</v>
-      </c>
-      <c r="K35" s="20"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A36" s="30"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="20"/>
-      <c r="J36" s="20"/>
-      <c r="K36" s="20"/>
-    </row>
-    <row r="37" spans="1:11" ht="33" x14ac:dyDescent="0.3">
-      <c r="A37" s="30">
-        <v>5</v>
-      </c>
-      <c r="B37" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
-      <c r="E37" s="20"/>
-      <c r="F37" s="20"/>
-      <c r="G37" s="20"/>
-      <c r="H37" s="20"/>
-      <c r="I37" s="20"/>
-      <c r="J37" s="20"/>
-      <c r="K37" s="20"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A38" s="30"/>
-      <c r="B38" s="31" t="str">
-        <f>B10</f>
-        <v>-for brick wall</v>
-      </c>
-      <c r="C38" s="32">
-        <v>1</v>
-      </c>
-      <c r="D38" s="33">
-        <f>D10</f>
-        <v>39.4</v>
-      </c>
-      <c r="E38" s="33">
-        <v>0.23</v>
-      </c>
-      <c r="F38" s="33">
-        <f>0.9+0.6-0.075*2</f>
-        <v>1.35</v>
-      </c>
-      <c r="G38" s="33">
-        <f>PRODUCT(C38:F38)</f>
-        <v>12.233700000000001</v>
-      </c>
-      <c r="H38" s="20"/>
-      <c r="I38" s="20"/>
-      <c r="J38" s="20"/>
-      <c r="K38" s="20"/>
-    </row>
-    <row r="39" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="8"/>
-      <c r="B39" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C39" s="10"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="13">
-        <f>SUM(G38:G38)</f>
-        <v>12.233700000000001</v>
-      </c>
-      <c r="H39" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I39" s="13">
-        <v>14491.84</v>
-      </c>
-      <c r="J39" s="15">
-        <f>G39*I39</f>
-        <v>177288.82300800001</v>
-      </c>
-      <c r="K39" s="12"/>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A40" s="30"/>
-      <c r="B40" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="20"/>
-      <c r="J40" s="15">
-        <f>0.13*G39*10374.74</f>
-        <v>16499.789375939999</v>
-      </c>
-      <c r="K40" s="20"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A41" s="30"/>
-      <c r="B41" s="34"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="20"/>
-      <c r="F41" s="20"/>
-      <c r="G41" s="20"/>
-      <c r="H41" s="20"/>
-      <c r="I41" s="20"/>
-      <c r="J41" s="15"/>
-      <c r="K41" s="20"/>
-    </row>
-    <row r="42" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
-      <c r="A42" s="8">
-        <v>6</v>
-      </c>
-      <c r="B42" s="35" t="s">
-        <v>37</v>
-      </c>
-      <c r="C42" s="10"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="12"/>
-      <c r="G42" s="40"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="13"/>
-      <c r="J42" s="40"/>
-      <c r="K42" s="12"/>
-    </row>
-    <row r="43" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="8"/>
-      <c r="B43" s="41" t="str">
-        <f>B28</f>
-        <v>-for brick wall</v>
-      </c>
-      <c r="C43" s="10">
-        <v>2</v>
-      </c>
-      <c r="D43" s="11">
-        <f>D38+C11*D11</f>
-        <v>45</v>
-      </c>
-      <c r="E43" s="12"/>
-      <c r="F43" s="12">
-        <v>0.9</v>
-      </c>
-      <c r="G43" s="42">
-        <f t="shared" ref="G43" si="1">PRODUCT(C43:F43)</f>
-        <v>81</v>
-      </c>
-      <c r="H43" s="14"/>
-      <c r="I43" s="13"/>
-      <c r="J43" s="40"/>
-      <c r="K43" s="12"/>
-    </row>
-    <row r="44" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="8"/>
-      <c r="B44" s="41" t="s">
-        <v>38</v>
-      </c>
-      <c r="C44" s="10"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
-      <c r="G44" s="40">
-        <f>SUM(G41:G43)</f>
-        <v>81</v>
-      </c>
-      <c r="H44" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="I44" s="13">
-        <v>415.5</v>
-      </c>
-      <c r="J44" s="40">
-        <f>G44*I44</f>
-        <v>33655.5</v>
-      </c>
-      <c r="K44" s="12"/>
-    </row>
-    <row r="45" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="8"/>
-      <c r="B45" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="C45" s="10"/>
-      <c r="D45" s="11"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="12"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="13"/>
-      <c r="J45" s="40">
-        <f>0.13*G44*11650.4/100</f>
-        <v>1226.7871200000002</v>
-      </c>
-      <c r="K45" s="12"/>
-    </row>
-    <row r="46" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
-      <c r="A46" s="8"/>
-      <c r="B46" s="39"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="11"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="12"/>
-      <c r="G46" s="40"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="13"/>
-      <c r="J46" s="40"/>
-      <c r="K46" s="12"/>
-    </row>
-    <row r="47" spans="1:11" s="16" customFormat="1" ht="32.4" x14ac:dyDescent="0.25">
-      <c r="A47" s="8">
-        <v>7</v>
-      </c>
-      <c r="B47" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="C47" s="10"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="40"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="13"/>
-      <c r="J47" s="40"/>
-      <c r="K47" s="12"/>
-    </row>
-    <row r="48" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="8"/>
-      <c r="B48" s="41" t="str">
-        <f>B43</f>
-        <v>-for brick wall</v>
-      </c>
-      <c r="C48" s="10">
-        <v>2</v>
-      </c>
-      <c r="D48" s="11">
-        <f>D43</f>
-        <v>45</v>
-      </c>
-      <c r="E48" s="12"/>
-      <c r="F48" s="12">
-        <v>0.9</v>
-      </c>
-      <c r="G48" s="42">
-        <f t="shared" ref="G48" si="2">PRODUCT(C48:F48)</f>
-        <v>81</v>
-      </c>
-      <c r="H48" s="14"/>
-      <c r="I48" s="13"/>
-      <c r="J48" s="40"/>
-      <c r="K48" s="12"/>
-    </row>
-    <row r="49" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="8"/>
-      <c r="B49" s="41" t="s">
-        <v>38</v>
-      </c>
-      <c r="C49" s="10"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="12"/>
-      <c r="F49" s="12"/>
-      <c r="G49" s="40">
-        <f>SUM(G46:G48)</f>
-        <v>81</v>
-      </c>
-      <c r="H49" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="I49" s="13">
-        <v>253.8</v>
-      </c>
-      <c r="J49" s="40">
-        <f>G49*I49</f>
-        <v>20557.8</v>
-      </c>
-      <c r="K49" s="12"/>
-    </row>
-    <row r="50" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="8"/>
-      <c r="B50" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="C50" s="10"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="12"/>
-      <c r="F50" s="12"/>
-      <c r="G50" s="40"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="13"/>
-      <c r="J50" s="40">
-        <f>0.13*G49*12736/100</f>
-        <v>1341.1008000000002</v>
-      </c>
-      <c r="K50" s="12"/>
-    </row>
-    <row r="51" spans="1:11" s="16" customFormat="1" ht="15" x14ac:dyDescent="0.3">
-      <c r="A51" s="8"/>
-      <c r="B51" s="39"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="12"/>
-      <c r="F51" s="12"/>
-      <c r="G51" s="40"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="13"/>
-      <c r="J51" s="40"/>
-      <c r="K51" s="12"/>
-    </row>
-    <row r="52" spans="1:11" ht="82.8" x14ac:dyDescent="0.3">
-      <c r="A52" s="30">
-        <v>8</v>
-      </c>
-      <c r="B52" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C52" s="20"/>
-      <c r="D52" s="20"/>
-      <c r="E52" s="20"/>
-      <c r="F52" s="20"/>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="20"/>
-      <c r="J52" s="20"/>
-      <c r="K52" s="20"/>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A53" s="30"/>
-      <c r="B53" s="31" t="str">
-        <f>B12</f>
-        <v>-for  stone masonary</v>
-      </c>
-      <c r="C53" s="32">
-        <v>1</v>
-      </c>
-      <c r="D53" s="33">
-        <f>D12</f>
-        <v>45</v>
-      </c>
-      <c r="E53" s="33">
-        <f>((F53/2)+0.45)/2</f>
-        <v>0.47499999999999998</v>
-      </c>
-      <c r="F53" s="33">
-        <v>1</v>
-      </c>
-      <c r="G53" s="33">
-        <f>PRODUCT(C53:F53)</f>
-        <v>21.375</v>
-      </c>
-      <c r="H53" s="20"/>
-      <c r="I53" s="20"/>
-      <c r="J53" s="20"/>
-      <c r="K53" s="20"/>
-    </row>
-    <row r="54" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="8"/>
-      <c r="B54" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C54" s="10"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="12"/>
-      <c r="F54" s="12"/>
-      <c r="G54" s="13">
-        <f>SUM(G53:G53)</f>
-        <v>21.375</v>
-      </c>
-      <c r="H54" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="I54" s="13">
-        <v>9878.43</v>
-      </c>
-      <c r="J54" s="15">
-        <f>G54*I54</f>
-        <v>211151.44125</v>
-      </c>
-      <c r="K54" s="12"/>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A55" s="30"/>
-      <c r="B55" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="20"/>
-      <c r="F55" s="20"/>
-      <c r="G55" s="20"/>
-      <c r="H55" s="20"/>
-      <c r="I55" s="20"/>
-      <c r="J55" s="15">
-        <f>0.13*G54*(27587.1)/5</f>
-        <v>15331.530825</v>
-      </c>
-      <c r="K55" s="20"/>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A56" s="30"/>
-      <c r="B56" s="20"/>
-      <c r="C56" s="20"/>
-      <c r="D56" s="20"/>
-      <c r="E56" s="20"/>
-      <c r="F56" s="20"/>
-      <c r="G56" s="20"/>
-      <c r="H56" s="20"/>
-      <c r="I56" s="20"/>
-      <c r="J56" s="20"/>
-      <c r="K56" s="20"/>
-    </row>
-    <row r="57" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="8">
-        <v>9</v>
-      </c>
-      <c r="B57" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C57" s="10">
-        <v>1</v>
-      </c>
-      <c r="D57" s="11"/>
-      <c r="E57" s="12"/>
-      <c r="F57" s="12"/>
-      <c r="G57" s="22">
-        <f t="shared" ref="G57" si="3">PRODUCT(C57:F57)</f>
-        <v>1</v>
-      </c>
-      <c r="H57" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="I57" s="13">
-        <v>500</v>
-      </c>
-      <c r="J57" s="22">
-        <f>G57*I57</f>
-        <v>500</v>
-      </c>
-      <c r="K57" s="12"/>
-    </row>
-    <row r="58" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="8"/>
-      <c r="B58" s="21"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="11"/>
-      <c r="E58" s="12"/>
-      <c r="F58" s="12"/>
-      <c r="G58" s="13"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="13"/>
-      <c r="J58" s="15"/>
-      <c r="K58" s="12"/>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A59" s="19"/>
-      <c r="B59" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="C59" s="29"/>
-      <c r="D59" s="18"/>
-      <c r="E59" s="18"/>
-      <c r="F59" s="18"/>
-      <c r="G59" s="15"/>
-      <c r="H59" s="15"/>
-      <c r="I59" s="15"/>
-      <c r="J59" s="15">
-        <f>SUM(J13:J57)</f>
-        <v>578400.81454687333</v>
-      </c>
-      <c r="K59" s="17"/>
-    </row>
-    <row r="61" spans="1:11" s="16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="23"/>
-      <c r="B61" s="37" t="s">
-        <v>22</v>
-      </c>
-      <c r="C61" s="43">
-        <f>J59</f>
-        <v>578400.81454687333</v>
-      </c>
-      <c r="D61" s="44"/>
-      <c r="E61" s="38">
-        <v>100</v>
-      </c>
-      <c r="F61" s="23"/>
-      <c r="G61" s="24"/>
-      <c r="H61" s="23"/>
-      <c r="I61" s="25"/>
-      <c r="J61" s="26"/>
-      <c r="K61" s="27"/>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B62" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="C62" s="49">
-        <v>500000</v>
-      </c>
-      <c r="D62" s="50"/>
-      <c r="E62" s="38"/>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B63" s="37" t="s">
-        <v>34</v>
-      </c>
-      <c r="C63" s="49">
-        <f>C62-C65-C66</f>
-        <v>475000</v>
-      </c>
-      <c r="D63" s="50"/>
-      <c r="E63" s="38">
-        <f>C63/C61*100</f>
-        <v>82.122982550106045</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B64" s="37" t="s">
-        <v>45</v>
-      </c>
-      <c r="C64" s="55">
-        <f>C61-C63</f>
-        <v>103400.81454687333</v>
-      </c>
-      <c r="D64" s="55"/>
-      <c r="E64" s="38">
-        <f>100-E63</f>
-        <v>17.877017449893955</v>
-      </c>
-    </row>
-    <row r="65" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B65" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="C65" s="43">
-        <f>C62*0.03</f>
-        <v>15000</v>
-      </c>
-      <c r="D65" s="44"/>
-      <c r="E65" s="38">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="66" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B66" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="C66" s="43">
-        <f>C62*0.02</f>
-        <v>10000</v>
-      </c>
-      <c r="D66" s="44"/>
-      <c r="E66" s="38">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="C62:D62"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="C64:D64"/>
-  </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
   <headerFooter>

</xml_diff>